<commit_message>
Added in error logging and cleaned up the console logging.
</commit_message>
<xml_diff>
--- a/example_data/metadata.xlsx
+++ b/example_data/metadata.xlsx
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -478,34 +478,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
+          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1907-24.2025</t>
+          <t>10.1523/JNEUROSCI.2378-24.2025</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Johanna B. Fritzinger</t>
+          <t>Keise Izuma</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>johanna_fritzinger@URMC.rochester.edu</t>
+          <t>izuma.keise@kochi-tech.ac.jp</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -515,34 +515,34 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Jocelyn M. Breton</t>
+          <t>Jae-Chang Kim</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>jo.breton@northeastern.edu</t>
+          <t>jaechang.kim@econ.uzh.ch</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Inbal Ben-Ami Bartal</t>
+          <t>Philippe N. Tobler</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -572,162 +572,162 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>inbalbe@tauex.tau.ac.il</t>
+          <t>phil.tobler@econ.uzh.ch</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
+          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0404-25.2025</t>
+          <t>10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Michael Vesia</t>
+          <t>Megan M. Davis</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>mvesia@umich.edu</t>
+          <t>davismeg@unc.edu</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ying Yu</t>
+          <t>Olivier Thoumine</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>yuying@tmu.edu.cn</t>
+          <t>olivier.thoumine@u-bordeaux.fr</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Qiang Liu</t>
+          <t>Xiaofen Zhong</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>qliu@tmu.edu.cn</t>
+          <t>zhongxf29@mail.sysu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Jie Zhou</t>
+          <t>Weixiang Guo</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>zhoujie@tmu.edu.cn</t>
+          <t>wxguo@genetics.ac.cn</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -737,165 +737,165 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A neural basis for distinguishing imagination from reality</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.015</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Nadine Dijkstra</t>
+          <t>Ying Yu</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>n.dijkstra@ucl.ac.uk</t>
+          <t>yuying@tmu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03398-0</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Francesca McEwan</t>
+          <t>Qiang Liu</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
+          <t>qliu@tmu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Jae-Chang Kim</t>
+          <t>Jie Zhou</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>jaechang.kim@econ.uzh.ch</t>
+          <t>zhoujie@tmu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Philippe N. Tobler</t>
+          <t>Wenjie Zhou</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>phil.tobler@econ.uzh.ch</t>
+          <t>zhouwj2022@shsmu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ethan B. Richman</t>
+          <t>Wenxi Huang</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -905,273 +905,273 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>deissero@stanford.edu?cc=vpbuch@stanford.edu&amp;amp;cc=cr2163@stanford.edu&amp;amp;cc=23sciencemag@pn.stanford.edu</t>
+          <t>tw.huang@siat.ac.cn</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Cephra Raja</t>
+          <t>Yuanyuan Liu</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>cr2163@stanford.edu</t>
+          <t>yuanyuan.liu@nih.gov</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1038/s41398-025-03322-6</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Vivek Buch</t>
+          <t>Ciyong Lu</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>vpbuch@stanford.edu</t>
+          <t>luciyong@mail.sysu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
+          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2218-24.2025</t>
+          <t>10.1038/s41398-025-03393-5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bin He</t>
+          <t>Chi-Yung Shang</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>bhe1@andrew.cmu.edu</t>
+          <t>cyshang@ntu.edu.tw</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
+          <t>A neural basis for distinguishing imagination from reality</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1139-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.015</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Paula T. Kuokkanen</t>
+          <t>Nadine Dijkstra</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>paula.kuokkanen@hu-berlin.de</t>
+          <t>n.dijkstra@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Karthik Srinivasan</t>
+          <t>Marie-Lucie Read</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>skarthik@mit.edu</t>
+          <t>readms2@cardiff.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Robert Desimone</t>
+          <t>Andrew D. Lawrence</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>desimone@mit.edu</t>
+          <t>Andrew.D.Lawrence@ed.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
+          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
+          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0491-25.2025</t>
+          <t>10.1038/s41398-025-03398-0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Barry J. Richmond</t>
+          <t>Francesca McEwan</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>barryrichmond@mail.nih.gov</t>
+          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1181,182 +1181,182 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
+          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2325-24.2025</t>
+          <t>10.1523/JNEUROSCI.1920-23.2025</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Martha E. Bickford</t>
+          <t>Adrianna C. Jenkins</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>martha.bickford@louisville.edu</t>
+          <t>acjenk@upenn.edu</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
+          <t>Grouping signals in primate visual cortex</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0436-25.2025</t>
+          <t>10.1016/j.neuron.2025.05.003</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Farran Briggs</t>
+          <t>Tom P. Franken</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>farran.briggs@nih.gov</t>
+          <t>ftom@wustl.edu</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1523/JNEUROSCI.1907-24.2025</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Wenjie Zhou</t>
+          <t>Johanna B. Fritzinger</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>zhouwj2022@shsmu.edu.cn</t>
+          <t>johanna_fritzinger@URMC.rochester.edu</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Wenxi Huang</t>
+          <t>Gina G. Turrigiano</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>tw.huang@siat.ac.cn</t>
+          <t>turrigiano@brandeis.edu</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1523/JNEUROSCI.0404-25.2025</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Yuanyuan Liu</t>
+          <t>Michael Vesia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>yuanyuan.liu@nih.gov</t>
+          <t>mvesia@umich.edu</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1366,165 +1366,165 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
+          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0044-25.2025</t>
+          <t>10.1523/JNEUROSCI.1139-24.2025</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bas Rokers</t>
+          <t>Paula T. Kuokkanen</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>rokers@nyu.edu</t>
+          <t>paula.kuokkanen@hu-berlin.de</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
+          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
+          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2411669122</t>
+          <t>10.1038/s41398-025-03401-8</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Olivier Thoumine</t>
+          <t>Andreas Walther</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>olivier.thoumine@u-bordeaux.fr</t>
+          <t>a.walther@psychologie.uzh.ch</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Grouping signals in primate visual cortex</t>
+          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.003</t>
+          <t>10.1523/JNEUROSCI.1920-24.2025</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Tom P. Franken</t>
+          <t>Alapakkam P. Sampath</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>ftom@wustl.edu</t>
+          <t>asampath@jsei.ucla.edu</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1523/JNEUROSCI.2218-24.2025</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Xiaodong Xu</t>
+          <t>Bin He</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>412alix@gmail.com</t>
+          <t>bhe1@andrew.cmu.edu</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1523/JNEUROSCI.0217-25.2025</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Lijuan Chen</t>
+          <t>Shinya Ohara</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1534,125 +1534,125 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>clj0430@126.com</t>
+          <t>shinya.ohara.d3@tohoku.ac.jp</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
+          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03393-5</t>
+          <t>10.1523/JNEUROSCI.0436-25.2025</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Chi-Yung Shang</t>
+          <t>Farran Briggs</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>cyshang@ntu.edu.tw</t>
+          <t>farran.briggs@nih.gov</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-23.2025</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Adrianna C. Jenkins</t>
+          <t>Christoph Bamberg</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>acjenk@upenn.edu</t>
+          <t>Christoph.bamberg@stud.plus.ac.at</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Yan Chen</t>
+          <t>Sarah Weigelt</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>chen_yan@hznu.edu.cn</t>
+          <t>sarah.weigelt@tu-dortmund.de</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1662,54 +1662,54 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1523/JNEUROSCI.2325-24.2025</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Haibo Di</t>
+          <t>Martha E. Bickford</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>haibodi@hznu.edu.cn</t>
+          <t>martha.bickford@louisville.edu</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Amy Hauck Newman</t>
+          <t>Stuart Berg</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1719,236 +1719,236 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>anewman@intra.nida.nih.gov</t>
+          <t>bergs@janelia.hhmi.org</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Zheng-Xiong Xi</t>
+          <t>Gerald M. Rubin</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>zxi@intra.nida.nih.gov</t>
+          <t>rubing@janelia.hhmi.org</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Xinzhong Dong</t>
+          <t>Michael B. Reiser</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>xdong2@jhmi.edu</t>
+          <t>reiserm@janelia.hhmi.org</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1523/JNEUROSCI.2187-24.2025</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Jun-Ming Zhang</t>
+          <t>Min Wu</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>jun-ming.zhang@uc.edu</t>
+          <t>min.wu@ndcn.ox.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Marie-Lucie Read</t>
+          <t>Wang Zheng</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>readms2@cardiff.ac.uk</t>
+          <t>wzheng86@wisc.edu</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Andrew D. Lawrence</t>
+          <t>Jeffrey R. Holt</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Andrew.D.Lawrence@ed.ac.uk</t>
+          <t>jeffrey.holt@childrens.harvard.edu</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
+          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03401-8</t>
+          <t>10.1523/JNEUROSCI.1114-24.2025</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Andreas Walther</t>
+          <t>Hackjin Kim</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>a.walther@psychologie.uzh.ch</t>
+          <t>hackjinkim@korea.ac.kr</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1958,17 +1958,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
+          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03272-z</t>
+          <t>10.1038/s41398-025-03399-z</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Froukje E. de Vries</t>
+          <t>Cristina Benatti</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1978,293 +1978,293 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>f.d.vries@nki.nl</t>
+          <t>cristina.benatti@unimore.it</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1876-24.2025</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Lidon Marin-Marin</t>
+          <t>Amy Hauck Newman</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>lidon.marinmarin@york.ac.uk</t>
+          <t>anewman@intra.nida.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Takahiro Morito</t>
+          <t>Zheng-Xiong Xi</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>takahiro.morito@riken.jp</t>
+          <t>zxi@intra.nida.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Takaomi C. Saido</t>
+          <t>Adam P. Caccavano</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>takaomi.saido@riken.jp</t>
+          <t>adam.caccavano@nih.gov</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2418176122</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Megan M. Davis</t>
+          <t>Kenneth A. Pelkey</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>davismeg@unc.edu</t>
+          <t>pelkeyk2@mail.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2187-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Min Wu</t>
+          <t>Chris J. McBain</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>min.wu@ndcn.ox.ac.uk</t>
+          <t>mcbainc@mail.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1523/JNEUROSCI.1788-24.2025</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Cong Liu</t>
+          <t>Mingzhou Ding</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>liulab@sioc.ac.cn</t>
+          <t>mding@bme.ufl.edu</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ShengQi Xiang</t>
+          <t>Karthik Srinivasan</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>cqxiang@ustc.edu.cn</t>
+          <t>skarthik@mit.edu</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Zhuohao He</t>
+          <t>Robert Desimone</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2274,14 +2274,14 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>hezh@sioc.ac.cn</t>
+          <t>desimone@mit.edu</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2291,34 +2291,34 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
+          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1001-24.2025</t>
+          <t>10.1523/JNEUROSCI.1876-24.2025</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Ekaterina Likhtik</t>
+          <t>Lidon Marin-Marin</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>elikhtik@genectr.hunter.cuny.edu</t>
+          <t>lidon.marinmarin@york.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2328,34 +2328,34 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Shigehiro Ohdo</t>
+          <t>Adam Steel</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>ohdo@phar.kyushu-u.ac.jp</t>
+          <t>adamdanielsteel@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2365,17 +2365,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Satoru Koyanagi</t>
+          <t>Caroline E. Robertson</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2385,162 +2385,162 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>koyanagi@phar.kyushu-u.ac.jp</t>
+          <t>cerw@dartmouth.edu</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
+          <t>Activity-dependent development of the body’s touch receptors</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03399-z</t>
+          <t>10.1016/j.neuron.2025.04.015</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Cristina Benatti</t>
+          <t>David D. Ginty</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>cristina.benatti@unimore.it</t>
+          <t>david_ginty@hms.harvard.edu</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-24.2025</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Alapakkam P. Sampath</t>
+          <t>Xiaodong Xu</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>asampath@jsei.ucla.edu</t>
+          <t>412alix@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.018</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Qingtao Sun</t>
+          <t>Lijuan Chen</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>qsun@cshl.edu</t>
+          <t>clj0430@126.com</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
+          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
+          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0217-25.2025</t>
+          <t>10.1038/s41398-025-03392-6</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Shinya Ohara</t>
+          <t>Christelle Langley</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>shinya.ohara.d3@tohoku.ac.jp</t>
+          <t>cl798@medschl.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2550,34 +2550,34 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1523/JNEUROSCI.0044-25.2025</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Adam Steel</t>
+          <t>Bas Rokers</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>adamdanielsteel@gmail.com</t>
+          <t>rokers@nyu.edu</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2587,34 +2587,34 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Caroline E. Robertson</t>
+          <t>Shigehiro Ohdo</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>cerw@dartmouth.edu</t>
+          <t>ohdo@phar.kyushu-u.ac.jp</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2624,17 +2624,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2378-24.2025</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Keise Izuma</t>
+          <t>Satoru Koyanagi</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2644,273 +2644,273 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>izuma.keise@kochi-tech.ac.jp</t>
+          <t>koyanagi@phar.kyushu-u.ac.jp</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1114-24.2025</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Hackjin Kim</t>
+          <t>Ethan B. Richman</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>hackjinkim@korea.ac.kr</t>
+          <t>deissero@stanford.edu?cc=vpbuch@stanford.edu&amp;amp;cc=cr2163@stanford.edu&amp;amp;cc=23sciencemag@pn.stanford.edu</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Xiaofen Zhong</t>
+          <t>Cephra Raja</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>zhongxf29@mail.sysu.edu.cn</t>
+          <t>cr2163@stanford.edu</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Weixiang Guo</t>
+          <t>Vivek Buch</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>wxguo@genetics.ac.cn</t>
+          <t>vpbuch@stanford.edu</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
+          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
+          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>10.1126/science.adt7705</t>
+          <t>10.1523/JNEUROSCI.1001-24.2025</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Yulong Li</t>
+          <t>Ekaterina Likhtik</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>yulongli@pku.edu.cn</t>
+          <t>elikhtik@genectr.hunter.cuny.edu</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Tilman Stephani</t>
+          <t>Lindsay A. Hohsfield</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>tilman.stephani@donders.ru.nl</t>
+          <t>lhohsfie@uci.edu</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Vadim V. Nikulin</t>
+          <t>Kim N. Green</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>nikulin@cbs.mpg.de</t>
+          <t>kngreen@uci.edu</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03390-8</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Ryan Smith</t>
+          <t>Yan Chen</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>rsmith@laureateinstitute.org</t>
+          <t>chen_yan@hznu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2920,17 +2920,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1788-24.2025</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Mingzhou Ding</t>
+          <t>Haibo Di</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2940,71 +2940,71 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>mding@bme.ufl.edu</t>
+          <t>haibodi@hznu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Activity-dependent development of the body’s touch receptors</t>
+          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.04.015</t>
+          <t>10.1523/JNEUROSCI.0491-25.2025</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>David D. Ginty</t>
+          <t>Barry J. Richmond</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>david_ginty@hms.harvard.edu</t>
+          <t>barryrichmond@mail.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03392-6</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Christelle Langley</t>
+          <t>Tilman Stephani</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3014,71 +3014,71 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>cl798@medschl.cam.ac.uk</t>
+          <t>tilman.stephani@donders.ru.nl</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Wang Zheng</t>
+          <t>Vadim V. Nikulin</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>wzheng86@wisc.edu</t>
+          <t>nikulin@cbs.mpg.de</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Jeffrey R. Holt</t>
+          <t>Yulong Li</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3088,88 +3088,88 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>jeffrey.holt@childrens.harvard.edu</t>
+          <t>yulongli@pku.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03322-6</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Ciyong Lu</t>
+          <t>Jocelyn M. Breton</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>luciyong@mail.sysu.edu.cn</t>
+          <t>jo.breton@northeastern.edu</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Lindsay A. Hohsfield</t>
+          <t>Inbal Ben-Ami Bartal</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>lhohsfie@uci.edu</t>
+          <t>inbalbe@tauex.tau.ac.il</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3179,71 +3179,71 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1016/j.neuron.2025.03.018</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Kim N. Green</t>
+          <t>Qingtao Sun</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>kngreen@uci.edu</t>
+          <t>qsun@cshl.edu</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
+          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2186-24.2025</t>
+          <t>10.1038/s41398-025-03272-z</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Siyi Chen (陈思佚)</t>
+          <t>Froukje E. de Vries</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Siyi.Chen@psy.lmu.de</t>
+          <t>f.d.vries@nki.nl</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3253,128 +3253,128 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Psychedelic control of neuroimmune interactions governing fear</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1038/s41586-025-08880-9</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Stuart Berg</t>
+          <t>Michael A. Wheeler</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>bergs@janelia.hhmi.org</t>
+          <t>mwheeler0@bwh.harvard.edu</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1038/s41398-025-03390-8</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Gerald M. Rubin</t>
+          <t>Ryan Smith</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>rubing@janelia.hhmi.org</t>
+          <t>rsmith@laureateinstitute.org</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Michael B. Reiser</t>
+          <t>Xinzhong Dong</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>reiserm@janelia.hhmi.org</t>
+          <t>xdong2@jhmi.edu</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2504775122</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Gina G. Turrigiano</t>
+          <t>Jun-Ming Zhang</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3384,88 +3384,88 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>turrigiano@brandeis.edu</t>
+          <t>jun-ming.zhang@uc.edu</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Christoph Bamberg</t>
+          <t>Cong Liu</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Christoph.bamberg@stud.plus.ac.at</t>
+          <t>liulab@sioc.ac.cn</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Sarah Weigelt</t>
+          <t>ShengQi Xiang</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>sarah.weigelt@tu-dortmund.de</t>
+          <t>cqxiang@ustc.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3475,138 +3475,138 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Adam P. Caccavano</t>
+          <t>Zhuohao He</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>adam.caccavano@nih.gov</t>
+          <t>hezh@sioc.ac.cn</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Kenneth A. Pelkey</t>
+          <t>Takahiro Morito</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>pelkeyk2@mail.nih.gov</t>
+          <t>takahiro.morito@riken.jp</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Chris J. McBain</t>
+          <t>Takaomi C. Saido</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>mcbainc@mail.nih.gov</t>
+          <t>takaomi.saido@riken.jp</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Psychedelic control of neuroimmune interactions governing fear</t>
+          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08880-9</t>
+          <t>10.1523/JNEUROSCI.2186-24.2025</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Michael A. Wheeler</t>
+          <t>Siyi Chen (陈思佚)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>mwheeler0@bwh.harvard.edu</t>
+          <t>Siyi.Chen@psy.lmu.de</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added coverage analysis script and results
</commit_message>
<xml_diff>
--- a/example_data/metadata.xlsx
+++ b/example_data/metadata.xlsx
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -478,27 +478,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2378-24.2025</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Keise Izuma</t>
+          <t>Jae-Chang Kim</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>izuma.keise@kochi-tech.ac.jp</t>
+          <t>jaechang.kim@econ.uzh.ch</t>
         </is>
       </c>
     </row>
@@ -525,24 +525,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Jae-Chang Kim</t>
+          <t>Philippe N. Tobler</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>jaechang.kim@econ.uzh.ch</t>
+          <t>phil.tobler@econ.uzh.ch</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1523/JNEUROSCI.0404-25.2025</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Philippe N. Tobler</t>
+          <t>Michael Vesia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -572,125 +572,125 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>phil.tobler@econ.uzh.ch</t>
+          <t>mvesia@umich.edu</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2418176122</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Megan M. Davis</t>
+          <t>Stuart Berg</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>davismeg@unc.edu</t>
+          <t>bergs@janelia.hhmi.org</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2411669122</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Olivier Thoumine</t>
+          <t>Gerald M. Rubin</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>olivier.thoumine@u-bordeaux.fr</t>
+          <t>rubing@janelia.hhmi.org</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Xiaofen Zhong</t>
+          <t>Michael B. Reiser</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>zhongxf29@mail.sysu.edu.cn</t>
+          <t>reiserm@janelia.hhmi.org</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -700,145 +700,145 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Weixiang Guo</t>
+          <t>Adam Steel</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>wxguo@genetics.ac.cn</t>
+          <t>adamdanielsteel@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Ying Yu</t>
+          <t>Caroline E. Robertson</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>yuying@tmu.edu.cn</t>
+          <t>cerw@dartmouth.edu</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.1907-24.2025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Qiang Liu</t>
+          <t>Johanna B. Fritzinger</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>qliu@tmu.edu.cn</t>
+          <t>johanna_fritzinger@URMC.rochester.edu</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.1920-24.2025</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Jie Zhou</t>
+          <t>Alapakkam P. Sampath</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>zhoujie@tmu.edu.cn</t>
+          <t>asampath@jsei.ucla.edu</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -848,219 +848,219 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Activity-dependent development of the body’s touch receptors</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1016/j.neuron.2025.04.015</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Wenjie Zhou</t>
+          <t>David D. Ginty</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>zhouwj2022@shsmu.edu.cn</t>
+          <t>david_ginty@hms.harvard.edu</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1523/JNEUROSCI.1788-24.2025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Wenxi Huang</t>
+          <t>Mingzhou Ding</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>tw.huang@siat.ac.cn</t>
+          <t>mding@bme.ufl.edu</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Psychedelic control of neuroimmune interactions governing fear</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1038/s41586-025-08880-9</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Yuanyuan Liu</t>
+          <t>Michael A. Wheeler</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>yuanyuan.liu@nih.gov</t>
+          <t>mwheeler0@bwh.harvard.edu</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
+          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03322-6</t>
+          <t>10.1523/JNEUROSCI.1139-24.2025</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ciyong Lu</t>
+          <t>Paula T. Kuokkanen</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>luciyong@mail.sysu.edu.cn</t>
+          <t>paula.kuokkanen@hu-berlin.de</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
+          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03393-5</t>
+          <t>10.1523/JNEUROSCI.0044-25.2025</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Chi-Yung Shang</t>
+          <t>Bas Rokers</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>cyshang@ntu.edu.tw</t>
+          <t>rokers@nyu.edu</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A neural basis for distinguishing imagination from reality</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.015</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Nadine Dijkstra</t>
+          <t>Tilman Stephani</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>n.dijkstra@ucl.ac.uk</t>
+          <t>tilman.stephani@donders.ru.nl</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1070,108 +1070,108 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Marie-Lucie Read</t>
+          <t>Vadim V. Nikulin</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>readms2@cardiff.ac.uk</t>
+          <t>nikulin@cbs.mpg.de</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>A neural basis for distinguishing imagination from reality</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.015</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Andrew D. Lawrence</t>
+          <t>Nadine Dijkstra</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Andrew.D.Lawrence@ed.ac.uk</t>
+          <t>n.dijkstra@ucl.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
+          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03398-0</t>
+          <t>10.1523/JNEUROSCI.1114-24.2025</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Francesca McEwan</t>
+          <t>Hackjin Kim</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
+          <t>hackjinkim@korea.ac.kr</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1181,17 +1181,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
+          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-23.2025</t>
+          <t>10.1523/JNEUROSCI.2378-24.2025</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Adrianna C. Jenkins</t>
+          <t>Keise Izuma</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1201,125 +1201,125 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>acjenk@upenn.edu</t>
+          <t>izuma.keise@kochi-tech.ac.jp</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Grouping signals in primate visual cortex</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.003</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Tom P. Franken</t>
+          <t>Xiaodong Xu</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>ftom@wustl.edu</t>
+          <t>412alix@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1907-24.2025</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Johanna B. Fritzinger</t>
+          <t>Lijuan Chen</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>johanna_fritzinger@URMC.rochester.edu</t>
+          <t>clj0430@126.com</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
+          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
+          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2504775122</t>
+          <t>10.1038/s41398-025-03272-z</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Gina G. Turrigiano</t>
+          <t>Froukje E. de Vries</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>turrigiano@brandeis.edu</t>
+          <t>f.d.vries@nki.nl</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1329,182 +1329,182 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
+          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0404-25.2025</t>
+          <t>10.1523/JNEUROSCI.2187-24.2025</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Michael Vesia</t>
+          <t>Min Wu</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>mvesia@umich.edu</t>
+          <t>min.wu@ndcn.ox.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1139-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Paula T. Kuokkanen</t>
+          <t>Xinzhong Dong</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>paula.kuokkanen@hu-berlin.de</t>
+          <t>xdong2@jhmi.edu</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03401-8</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Andreas Walther</t>
+          <t>Jun-Ming Zhang</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>a.walther@psychologie.uzh.ch</t>
+          <t>jun-ming.zhang@uc.edu</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-24.2025</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Alapakkam P. Sampath</t>
+          <t>Karthik Srinivasan</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>asampath@jsei.ucla.edu</t>
+          <t>skarthik@mit.edu</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2218-24.2025</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bin He</t>
+          <t>Robert Desimone</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>bhe1@andrew.cmu.edu</t>
+          <t>desimone@mit.edu</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1514,17 +1514,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
+          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0217-25.2025</t>
+          <t>10.1523/JNEUROSCI.1001-24.2025</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Shinya Ohara</t>
+          <t>Ekaterina Likhtik</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1534,219 +1534,219 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>shinya.ohara.d3@tohoku.ac.jp</t>
+          <t>elikhtik@genectr.hunter.cuny.edu</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
+          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0436-25.2025</t>
+          <t>10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Farran Briggs</t>
+          <t>Yulong Li</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>farran.briggs@nih.gov</t>
+          <t>yulongli@pku.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1523/JNEUROSCI.2218-24.2025</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Christoph Bamberg</t>
+          <t>Bin He</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Christoph.bamberg@stud.plus.ac.at</t>
+          <t>bhe1@andrew.cmu.edu</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Sarah Weigelt</t>
+          <t>Wenjie Zhou</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>sarah.weigelt@tu-dortmund.de</t>
+          <t>zhouwj2022@shsmu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2325-24.2025</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Martha E. Bickford</t>
+          <t>Wenxi Huang</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>martha.bickford@louisville.edu</t>
+          <t>tw.huang@siat.ac.cn</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Stuart Berg</t>
+          <t>Yuanyuan Liu</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>bergs@janelia.hhmi.org</t>
+          <t>yuanyuan.liu@nih.gov</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1038/s41398-025-03393-5</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Gerald M. Rubin</t>
+          <t>Chi-Yung Shang</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1756,88 +1756,88 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>rubing@janelia.hhmi.org</t>
+          <t>cyshang@ntu.edu.tw</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Michael B. Reiser</t>
+          <t>Gina G. Turrigiano</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>reiserm@janelia.hhmi.org</t>
+          <t>turrigiano@brandeis.edu</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
+          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2187-24.2025</t>
+          <t>10.1038/s41398-025-03399-z</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Min Wu</t>
+          <t>Cristina Benatti</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>min.wu@ndcn.ox.ac.uk</t>
+          <t>cristina.benatti@unimore.it</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1847,17 +1847,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Wang Zheng</t>
+          <t>Adam P. Caccavano</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1867,14 +1867,14 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>wzheng86@wisc.edu</t>
+          <t>adam.caccavano@nih.gov</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1884,91 +1884,91 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Jeffrey R. Holt</t>
+          <t>Kenneth A. Pelkey</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>jeffrey.holt@childrens.harvard.edu</t>
+          <t>pelkeyk2@mail.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1114-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Hackjin Kim</t>
+          <t>Chris J. McBain</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>hackjinkim@korea.ac.kr</t>
+          <t>mcbainc@mail.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
+          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03399-z</t>
+          <t>10.1523/JNEUROSCI.0491-25.2025</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Cristina Benatti</t>
+          <t>Barry J. Richmond</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1978,162 +1978,162 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>cristina.benatti@unimore.it</t>
+          <t>barryrichmond@mail.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Amy Hauck Newman</t>
+          <t>Ethan B. Richman</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>anewman@intra.nida.nih.gov</t>
+          <t>deissero@stanford.edu?cc=vpbuch@stanford.edu&amp;amp;cc=cr2163@stanford.edu&amp;amp;cc=23sciencemag@pn.stanford.edu</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Zheng-Xiong Xi</t>
+          <t>Cephra Raja</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>zxi@intra.nida.nih.gov</t>
+          <t>cr2163@stanford.edu</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Adam P. Caccavano</t>
+          <t>Vivek Buch</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>adam.caccavano@nih.gov</t>
+          <t>vpbuch@stanford.edu</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1038/s41398-025-03392-6</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Kenneth A. Pelkey</t>
+          <t>Christelle Langley</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>pelkeyk2@mail.nih.gov</t>
+          <t>cl798@medschl.cam.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2143,34 +2143,34 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Grouping signals in primate visual cortex</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1016/j.neuron.2025.05.003</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Chris J. McBain</t>
+          <t>Tom P. Franken</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>mcbainc@mail.nih.gov</t>
+          <t>ftom@wustl.edu</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2180,313 +2180,313 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
+          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1788-24.2025</t>
+          <t>10.1523/JNEUROSCI.1876-24.2025</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mingzhou Ding</t>
+          <t>Lidon Marin-Marin</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>mding@bme.ufl.edu</t>
+          <t>lidon.marinmarin@york.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Karthik Srinivasan</t>
+          <t>Xiaofen Zhong</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>skarthik@mit.edu</t>
+          <t>zhongxf29@mail.sysu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Robert Desimone</t>
+          <t>Weixiang Guo</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>desimone@mit.edu</t>
+          <t>wxguo@genetics.ac.cn</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
+          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1876-24.2025</t>
+          <t>10.1038/s41398-025-03322-6</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Lidon Marin-Marin</t>
+          <t>Ciyong Lu</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>lidon.marinmarin@york.ac.uk</t>
+          <t>luciyong@mail.sysu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Adam Steel</t>
+          <t>Wang Zheng</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>adamdanielsteel@gmail.com</t>
+          <t>wzheng86@wisc.edu</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Caroline E. Robertson</t>
+          <t>Jeffrey R. Holt</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>cerw@dartmouth.edu</t>
+          <t>jeffrey.holt@childrens.harvard.edu</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Activity-dependent development of the body’s touch receptors</t>
+          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.04.015</t>
+          <t>10.1523/JNEUROSCI.2186-24.2025</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>David D. Ginty</t>
+          <t>Siyi Chen (陈思佚)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>david_ginty@hms.harvard.edu</t>
+          <t>Siyi.Chen@psy.lmu.de</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Xiaodong Xu</t>
+          <t>Shigehiro Ohdo</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>412alix@gmail.com</t>
+          <t>ohdo@phar.kyushu-u.ac.jp</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Lijuan Chen</t>
+          <t>Satoru Koyanagi</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2496,182 +2496,182 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>clj0430@126.com</t>
+          <t>koyanagi@phar.kyushu-u.ac.jp</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03392-6</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Christelle Langley</t>
+          <t>Ying Yu</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>cl798@medschl.cam.ac.uk</t>
+          <t>yuying@tmu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0044-25.2025</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Bas Rokers</t>
+          <t>Qiang Liu</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>rokers@nyu.edu</t>
+          <t>qliu@tmu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Shigehiro Ohdo</t>
+          <t>Jie Zhou</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>ohdo@phar.kyushu-u.ac.jp</t>
+          <t>zhoujie@tmu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.018</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Satoru Koyanagi</t>
+          <t>Qingtao Sun</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>koyanagi@phar.kyushu-u.ac.jp</t>
+          <t>qsun@cshl.edu</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Ethan B. Richman</t>
+          <t>Cong Liu</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2681,34 +2681,34 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>deissero@stanford.edu?cc=vpbuch@stanford.edu&amp;amp;cc=cr2163@stanford.edu&amp;amp;cc=23sciencemag@pn.stanford.edu</t>
+          <t>liulab@sioc.ac.cn</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Cephra Raja</t>
+          <t>ShengQi Xiang</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2718,81 +2718,81 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>cr2163@stanford.edu</t>
+          <t>cqxiang@ustc.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Vivek Buch</t>
+          <t>Zhuohao He</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>vpbuch@stanford.edu</t>
+          <t>hezh@sioc.ac.cn</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1001-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Ekaterina Likhtik</t>
+          <t>Lindsay A. Hohsfield</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>elikhtik@genectr.hunter.cuny.edu</t>
+          <t>lhohsfie@uci.edu</t>
         </is>
       </c>
     </row>
@@ -2819,61 +2819,61 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Lindsay A. Hohsfield</t>
+          <t>Kim N. Green</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>lhohsfie@uci.edu</t>
+          <t>kngreen@uci.edu</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Kim N. Green</t>
+          <t>Takahiro Morito</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>kngreen@uci.edu</t>
+          <t>takahiro.morito@riken.jp</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2883,71 +2883,71 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Yan Chen</t>
+          <t>Takaomi C. Saido</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>chen_yan@hznu.edu.cn</t>
+          <t>takaomi.saido@riken.jp</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Haibo Di</t>
+          <t>Megan M. Davis</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>haibodi@hznu.edu.cn</t>
+          <t>davismeg@unc.edu</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2957,34 +2957,34 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0491-25.2025</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Barry J. Richmond</t>
+          <t>Jocelyn M. Breton</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>barryrichmond@mail.nih.gov</t>
+          <t>jo.breton@northeastern.edu</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2994,108 +2994,108 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Tilman Stephani</t>
+          <t>Inbal Ben-Ami Bartal</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>tilman.stephani@donders.ru.nl</t>
+          <t>inbalbe@tauex.tau.ac.il</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Vadim V. Nikulin</t>
+          <t>Amy Hauck Newman</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>nikulin@cbs.mpg.de</t>
+          <t>anewman@intra.nida.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>10.1126/science.adt7705</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Yulong Li</t>
+          <t>Zheng-Xiong Xi</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>yulongli@pku.edu.cn</t>
+          <t>zxi@intra.nida.nih.gov</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3105,202 +3105,202 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1523/JNEUROSCI.0217-25.2025</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Jocelyn M. Breton</t>
+          <t>Shinya Ohara</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>jo.breton@northeastern.edu</t>
+          <t>shinya.ohara.d3@tohoku.ac.jp</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1038/s41398-025-03401-8</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Inbal Ben-Ami Bartal</t>
+          <t>Andreas Walther</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>inbalbe@tauex.tau.ac.il</t>
+          <t>a.walther@psychologie.uzh.ch</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.018</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Qingtao Sun</t>
+          <t>Christoph Bamberg</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>qsun@cshl.edu</t>
+          <t>Christoph.bamberg@stud.plus.ac.at</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03272-z</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Froukje E. de Vries</t>
+          <t>Sarah Weigelt</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>f.d.vries@nki.nl</t>
+          <t>sarah.weigelt@tu-dortmund.de</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Psychedelic control of neuroimmune interactions governing fear</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08880-9</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Michael A. Wheeler</t>
+          <t>Yan Chen</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>mwheeler0@bwh.harvard.edu</t>
+          <t>chen_yan@hznu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03390-8</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Ryan Smith</t>
+          <t>Haibo Di</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -3310,199 +3310,199 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>rsmith@laureateinstitute.org</t>
+          <t>haibodi@hznu.edu.cn</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1523/JNEUROSCI.1920-23.2025</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Xinzhong Dong</t>
+          <t>Adrianna C. Jenkins</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>xdong2@jhmi.edu</t>
+          <t>acjenk@upenn.edu</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Jun-Ming Zhang</t>
+          <t>Marie-Lucie Read</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>jun-ming.zhang@uc.edu</t>
+          <t>readms2@cardiff.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Cong Liu</t>
+          <t>Andrew D. Lawrence</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>liulab@sioc.ac.cn</t>
+          <t>Andrew.D.Lawrence@ed.ac.uk</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ShengQi Xiang</t>
+          <t>Olivier Thoumine</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>cqxiang@ustc.edu.cn</t>
+          <t>olivier.thoumine@u-bordeaux.fr</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1038/s41398-025-03390-8</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Zhuohao He</t>
+          <t>Ryan Smith</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>hezh@sioc.ac.cn</t>
+          <t>rsmith@laureateinstitute.org</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3512,34 +3512,34 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1523/JNEUROSCI.2325-24.2025</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Takahiro Morito</t>
+          <t>Martha E. Bickford</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>takahiro.morito@riken.jp</t>
+          <t>martha.bickford@louisville.edu</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3549,17 +3549,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1523/JNEUROSCI.0436-25.2025</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Takaomi C. Saido</t>
+          <t>Farran Briggs</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3569,44 +3569,44 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>takaomi.saido@riken.jp</t>
+          <t>farran.briggs@nih.gov</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
+          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2186-24.2025</t>
+          <t>10.1038/s41398-025-03398-0</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Siyi Chen (陈思佚)</t>
+          <t>Francesca McEwan</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Siyi.Chen@psy.lmu.de</t>
+          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added validation function for the extraction process. Manualyl extracted ground truth metadata. Attempted to fix minor issues in extraction.
</commit_message>
<xml_diff>
--- a/example_data/metadata.xlsx
+++ b/example_data/metadata.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,11 +464,16 @@
           <t>author_email</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>match_method</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -478,71 +483,81 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1523/JNEUROSCI.1001-24.2025</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Jae-Chang Kim</t>
+          <t>Ekaterina Likhtik</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>jaechang.kim@econ.uzh.ch</t>
+          <t>elikhtik@genectr.hunter.cuny.edu</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1038/s41398-025-03401-8</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Philippe N. Tobler</t>
+          <t>Andreas Walther</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>phil.tobler@econ.uzh.ch</t>
+          <t>a.walther@psychologie.uzh.ch</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -552,128 +567,143 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0404-25.2025</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Michael Vesia</t>
+          <t>Tilman Stephani</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>mvesia@umich.edu</t>
+          <t>tilman.stephani@donders.ru.nl</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Stuart Berg</t>
+          <t>Vadim V. Nikulin</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>bergs@janelia.hhmi.org</t>
+          <t>nikulin@cbs.mpg.de</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1038/s41398-025-03322-6</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Gerald M. Rubin</t>
+          <t>Ciyong Lu</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>rubing@janelia.hhmi.org</t>
+          <t>luciyong@mail.sysu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1523/JNEUROSCI.2378-24.2025</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Michael B. Reiser</t>
+          <t>Keise Izuma</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -683,14 +713,19 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>reiserm@janelia.hhmi.org</t>
+          <t>izuma.keise@kochi-tech.ac.jp</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -700,34 +735,39 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Adam Steel</t>
+          <t>Xiaofen Zhong</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>adamdanielsteel@gmail.com</t>
+          <t>zhongxf29@mail.sysu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -737,17 +777,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Caroline E. Robertson</t>
+          <t>Weixiang Guo</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -757,14 +797,19 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>cerw@dartmouth.edu</t>
+          <t>wxguo@genetics.ac.cn</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -774,71 +819,81 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
+          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1907-24.2025</t>
+          <t>10.1523/JNEUROSCI.2218-24.2025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Johanna B. Fritzinger</t>
+          <t>Bin He</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>johanna_fritzinger@URMC.rochester.edu</t>
+          <t>bhe1@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Alapakkam P. Sampath</t>
+          <t>Xinzhong Dong</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>asampath@jsei.ucla.edu</t>
+          <t>xdong2@jhmi.edu</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -848,17 +903,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Activity-dependent development of the body’s touch receptors</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.04.015</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>David D. Ginty</t>
+          <t>Jun-Ming Zhang</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -868,88 +923,103 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>david_ginty@hms.harvard.edu</t>
+          <t>jun-ming.zhang@uc.edu</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
+          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1788-24.2025</t>
+          <t>10.1038/s41398-025-03393-5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Mingzhou Ding</t>
+          <t>Chi-Yung Shang</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>mding@bme.ufl.edu</t>
+          <t>cyshang@ntu.edu.tw</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Psychedelic control of neuroimmune interactions governing fear</t>
+          <t>Grouping signals in primate visual cortex</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08880-9</t>
+          <t>10.1016/j.neuron.2025.05.003</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Michael A. Wheeler</t>
+          <t>Tom P. Franken</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>mwheeler0@bwh.harvard.edu</t>
+          <t>ftom@wustl.edu</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -959,17 +1029,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
+          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1139-24.2025</t>
+          <t>10.1523/JNEUROSCI.2187-24.2025</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Paula T. Kuokkanen</t>
+          <t>Min Wu</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -979,162 +1049,187 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>paula.kuokkanen@hu-berlin.de</t>
+          <t>min.wu@ndcn.ox.ac.uk</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0044-25.2025</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bas Rokers</t>
+          <t>Christoph Bamberg</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>rokers@nyu.edu</t>
+          <t>Christoph.bamberg@stud.plus.ac.at</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tilman Stephani</t>
+          <t>Sarah Weigelt</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>tilman.stephani@donders.ru.nl</t>
+          <t>sarah.weigelt@tu-dortmund.de</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Vadim V. Nikulin</t>
+          <t>Xiaodong Xu</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nikulin@cbs.mpg.de</t>
+          <t>412alix@gmail.com</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>proximity</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A neural basis for distinguishing imagination from reality</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.015</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Nadine Dijkstra</t>
+          <t>Lijuan Chen</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>n.dijkstra@ucl.ac.uk</t>
+          <t>clj0430@126.com</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>proximity</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1144,17 +1239,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
+          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1114-24.2025</t>
+          <t>10.1523/JNEUROSCI.0404-25.2025</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Hackjin Kim</t>
+          <t>Michael Vesia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1164,108 +1259,123 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>hackjinkim@korea.ac.kr</t>
+          <t>mvesia@umich.edu</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2378-24.2025</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Keise Izuma</t>
+          <t>Karthik Srinivasan</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>izuma.keise@kochi-tech.ac.jp</t>
+          <t>skarthik@mit.edu</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Xiaodong Xu</t>
+          <t>Robert Desimone</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>412alix@gmail.com</t>
+          <t>desimone@mit.edu</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1523/JNEUROSCI.1920-24.2025</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Lijuan Chen</t>
+          <t>Alapakkam P. Sampath</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1275,162 +1385,187 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>clj0430@126.com</t>
+          <t>asampath@jsei.ucla.edu</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03272-z</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Froukje E. de Vries</t>
+          <t>Lindsay A. Hohsfield</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>f.d.vries@nki.nl</t>
+          <t>lhohsfie@uci.edu</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2187-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Min Wu</t>
+          <t>Kim N. Green</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>min.wu@ndcn.ox.ac.uk</t>
+          <t>kngreen@uci.edu</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1523/JNEUROSCI.1876-24.2025</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Xinzhong Dong</t>
+          <t>Lidon Marin-Marin</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>xdong2@jhmi.edu</t>
+          <t>lidon.marinmarin@york.ac.uk</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Jun-Ming Zhang</t>
+          <t>Megan M. Davis</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>jun-ming.zhang@uc.edu</t>
+          <t>davismeg@unc.edu</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1440,71 +1575,81 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Karthik Srinivasan</t>
+          <t>Olivier Thoumine</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>skarthik@mit.edu</t>
+          <t>olivier.thoumine@u-bordeaux.fr</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1523/JNEUROSCI.1788-24.2025</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Robert Desimone</t>
+          <t>Mingzhou Ding</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>desimone@mit.edu</t>
+          <t>mding@bme.ufl.edu</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1514,17 +1659,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
+          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1001-24.2025</t>
+          <t>10.1523/JNEUROSCI.0044-25.2025</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Ekaterina Likhtik</t>
+          <t>Bas Rokers</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1534,51 +1679,61 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>elikhtik@genectr.hunter.cuny.edu</t>
+          <t>rokers@nyu.edu</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
+          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
+          <t>Psychedelic control of neuroimmune interactions governing fear</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10.1126/science.adt7705</t>
+          <t>10.1038/s41586-025-08880-9</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Yulong Li</t>
+          <t>Michael A. Wheeler</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>yulongli@pku.edu.cn</t>
+          <t>mwheeler0@bwh.harvard.edu</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1588,256 +1743,291 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
+          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2218-24.2025</t>
+          <t>10.1523/JNEUROSCI.2186-24.2025</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Bin He</t>
+          <t>Siyi Chen (陈思佚)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>bhe1@andrew.cmu.edu</t>
+          <t>Siyi.Chen@psy.lmu.de</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1523/JNEUROSCI.0217-25.2025</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Wenjie Zhou</t>
+          <t>Shinya Ohara</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>zhouwj2022@shsmu.edu.cn</t>
+          <t>shinya.ohara.d3@tohoku.ac.jp</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Wenxi Huang</t>
+          <t>Stuart Berg</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>tw.huang@siat.ac.cn</t>
+          <t>bergs@janelia.hhmi.org</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Yuanyuan Liu</t>
+          <t>Gerald M. Rubin</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>yuanyuan.liu@nih.gov</t>
+          <t>rubing@janelia.hhmi.org</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03393-5</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Chi-Yung Shang</t>
+          <t>Michael B. Reiser</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>cyshang@ntu.edu.tw</t>
+          <t>reiserm@janelia.hhmi.org</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2504775122</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Gina G. Turrigiano</t>
+          <t>Ying Yu</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>turrigiano@brandeis.edu</t>
+          <t>yuying@tmu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03399-z</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Cristina Benatti</t>
+          <t>Qiang Liu</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>cristina.benatti@unimore.it</t>
+          <t>qliu@tmu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1847,293 +2037,333 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Adam P. Caccavano</t>
+          <t>Jie Zhou</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>adam.caccavano@nih.gov</t>
+          <t>zhoujie@tmu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Kenneth A. Pelkey</t>
+          <t>Yan Chen</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>pelkeyk2@mail.nih.gov</t>
+          <t>chen_yan@hznu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Chris J. McBain</t>
+          <t>Haibo Di</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>mcbainc@mail.nih.gov</t>
+          <t>haibodi@hznu.edu.cn</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
+          <t>A neural basis for distinguishing imagination from reality</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0491-25.2025</t>
+          <t>10.1016/j.neuron.2025.05.015</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Barry J. Richmond</t>
+          <t>Nadine Dijkstra</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>barryrichmond@mail.nih.gov</t>
+          <t>n.dijkstra@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Activity-dependent development of the body’s touch receptors</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1016/j.neuron.2025.04.015</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Ethan B. Richman</t>
+          <t>David D. Ginty</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>deissero@stanford.edu?cc=vpbuch@stanford.edu&amp;amp;cc=cr2163@stanford.edu&amp;amp;cc=23sciencemag@pn.stanford.edu</t>
+          <t>david_ginty@hms.harvard.edu</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1523/JNEUROSCI.1139-24.2025</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Cephra Raja</t>
+          <t>Paula T. Kuokkanen</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>cr2163@stanford.edu</t>
+          <t>paula.kuokkanen@hu-berlin.de</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Vivek Buch</t>
+          <t>Shigehiro Ohdo</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>vpbuch@stanford.edu</t>
+          <t>ohdo@phar.kyushu-u.ac.jp</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03392-6</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Christelle Langley</t>
+          <t>Satoru Koyanagi</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>cl798@medschl.cam.ac.uk</t>
+          <t>koyanagi@phar.kyushu-u.ac.jp</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2143,256 +2373,291 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Grouping signals in primate visual cortex</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.003</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Tom P. Franken</t>
+          <t>Cong Liu</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>ftom@wustl.edu</t>
+          <t>liulab@sioc.ac.cn</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1876-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Lidon Marin-Marin</t>
+          <t>ShengQi Xiang</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>lidon.marinmarin@york.ac.uk</t>
+          <t>cqxiang@ustc.edu.cn</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Xiaofen Zhong</t>
+          <t>Zhuohao He</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>zhongxf29@mail.sysu.edu.cn</t>
+          <t>hezh@sioc.ac.cn</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Weixiang Guo</t>
+          <t>Gina G. Turrigiano</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>wxguo@genetics.ac.cn</t>
+          <t>turrigiano@brandeis.edu</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03322-6</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Ciyong Lu</t>
+          <t>Jae-Chang Kim</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>luciyong@mail.sysu.edu.cn</t>
+          <t>jaechang.kim@econ.uzh.ch</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Wang Zheng</t>
+          <t>Philippe N. Tobler</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>wzheng86@wisc.edu</t>
+          <t>phil.tobler@econ.uzh.ch</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1523/JNEUROSCI.1907-24.2025</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Jeffrey R. Holt</t>
+          <t>Johanna B. Fritzinger</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>jeffrey.holt@childrens.harvard.edu</t>
+          <t>johanna_fritzinger@URMC.rochester.edu</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2402,34 +2667,39 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
+          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2186-24.2025</t>
+          <t>10.1523/JNEUROSCI.2325-24.2025</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Siyi Chen (陈思佚)</t>
+          <t>Martha E. Bickford</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Siyi.Chen@psy.lmu.de</t>
+          <t>martha.bickford@louisville.edu</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2439,17 +2709,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Shigehiro Ohdo</t>
+          <t>Jocelyn M. Breton</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2459,14 +2729,19 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>ohdo@phar.kyushu-u.ac.jp</t>
+          <t>jo.breton@northeastern.edu</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2476,17 +2751,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Satoru Koyanagi</t>
+          <t>Inbal Ben-Ami Bartal</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2496,14 +2771,19 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>koyanagi@phar.kyushu-u.ac.jp</t>
+          <t>inbalbe@tauex.tau.ac.il</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2513,498 +2793,563 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1016/j.neuron.2025.03.018</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Ying Yu</t>
+          <t>Qingtao Sun</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>yuying@tmu.edu.cn</t>
+          <t>qsun@cshl.edu</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.1920-23.2025</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Qiang Liu</t>
+          <t>Adrianna C. Jenkins</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>qliu@tmu.edu.cn</t>
+          <t>acjenk@upenn.edu</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1038/s41398-025-03399-z</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Jie Zhou</t>
+          <t>Cristina Benatti</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>zhoujie@tmu.edu.cn</t>
+          <t>cristina.benatti@unimore.it</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
+          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.018</t>
+          <t>10.1038/s41398-025-03392-6</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Qingtao Sun</t>
+          <t>Christelle Langley</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>qsun@cshl.edu</t>
+          <t>cl798@medschl.cam.ac.uk</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1523/JNEUROSCI.0491-25.2025</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Cong Liu</t>
+          <t>Barry J. Richmond</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>liulab@sioc.ac.cn</t>
+          <t>barryrichmond@mail.nih.gov</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ShengQi Xiang</t>
+          <t>Amy Hauck Newman</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>cqxiang@ustc.edu.cn</t>
+          <t>anewman@intra.nida.nih.gov</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Zhuohao He</t>
+          <t>Zheng-Xiong Xi</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>hezh@sioc.ac.cn</t>
+          <t>zxi@intra.nida.nih.gov</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1038/s41398-025-03390-8</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Lindsay A. Hohsfield</t>
+          <t>Ryan Smith</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>lhohsfie@uci.edu</t>
+          <t>rsmith@laureateinstitute.org</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Kim N. Green</t>
+          <t>Ethan B. Richman</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>kngreen@uci.edu</t>
+          <t>deissero@stanford.edu</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Takahiro Morito</t>
+          <t>Cephra Raja</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>takahiro.morito@riken.jp</t>
+          <t>cr2163@stanford.edu</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Takaomi C. Saido</t>
+          <t>Vivek Buch</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>takaomi.saido@riken.jp</t>
+          <t>vpbuch@stanford.edu</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2418176122</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Megan M. Davis</t>
+          <t>Karl Deisseroth</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>davismeg@unc.edu</t>
+          <t>deissero@stanford.edu?cc=vpbuch@stanford.edu&amp;amp;cc=cr2163@stanford.edu&amp;amp;cc=23sciencemag@pn.stanford.edu</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1038/s41398-025-03398-0</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Jocelyn M. Breton</t>
+          <t>Francesca McEwan</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>jo.breton@northeastern.edu</t>
+          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1038/s41398-025-03272-z</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Inbal Ben-Ami Bartal</t>
+          <t>Froukje E. de Vries</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3014,273 +3359,313 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>inbalbe@tauex.tau.ac.il</t>
+          <t>f.d.vries@nki.nl</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1523/JNEUROSCI.0436-25.2025</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Amy Hauck Newman</t>
+          <t>Farran Briggs</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>anewman@intra.nida.nih.gov</t>
+          <t>farran.briggs@nih.gov</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Zheng-Xiong Xi</t>
+          <t>Adam P. Caccavano</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>zxi@intra.nida.nih.gov</t>
+          <t>adam.caccavano@nih.gov</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0217-25.2025</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Shinya Ohara</t>
+          <t>Kenneth A. Pelkey</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>shinya.ohara.d3@tohoku.ac.jp</t>
+          <t>pelkeyk2@mail.nih.gov</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03401-8</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Andreas Walther</t>
+          <t>Chris J. McBain</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>a.walther@psychologie.uzh.ch</t>
+          <t>mcbainc@mail.nih.gov</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Christoph Bamberg</t>
+          <t>Wang Zheng</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Christoph.bamberg@stud.plus.ac.at</t>
+          <t>wzheng86@wisc.edu</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Sarah Weigelt</t>
+          <t>Jeffrey R. Holt</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>sarah.weigelt@tu-dortmund.de</t>
+          <t>jeffrey.holt@childrens.harvard.edu</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Yan Chen</t>
+          <t>Yulong Li</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>chen_yan@hznu.edu.cn</t>
+          <t>yulongli@pku.edu.cn</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3290,34 +3675,39 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Haibo Di</t>
+          <t>Marie-Lucie Read</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>haibodi@hznu.edu.cn</t>
+          <t>readms2@cardiff.ac.uk</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3327,34 +3717,39 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-23.2025</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Adrianna C. Jenkins</t>
+          <t>Andrew D. Lawrence</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>acjenk@upenn.edu</t>
+          <t>Andrew.D.Lawrence@ed.ac.uk</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3364,17 +3759,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Marie-Lucie Read</t>
+          <t>Adam Steel</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3384,14 +3779,19 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>readms2@cardiff.ac.uk</t>
+          <t>adamdanielsteel@gmail.com</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3401,91 +3801,101 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Andrew D. Lawrence</t>
+          <t>Caroline E. Robertson</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Andrew.D.Lawrence@ed.ac.uk</t>
+          <t>cerw@dartmouth.edu</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>proximity</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2411669122</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Olivier Thoumine</t>
+          <t>Takahiro Morito</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>olivier.thoumine@u-bordeaux.fr</t>
+          <t>takahiro.morito@riken.jp</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03390-8</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Ryan Smith</t>
+          <t>Takaomi C. Saido</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3495,14 +3905,19 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>rsmith@laureateinstitute.org</t>
+          <t>takaomi.saido@riken.jp</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3512,101 +3927,32 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
+          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2325-24.2025</t>
+          <t>10.1523/JNEUROSCI.1114-24.2025</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Martha E. Bickford</t>
+          <t>Hackjin Kim</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>martha.bickford@louisville.edu</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>The Journal of Neuroscience</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>10.1523/JNEUROSCI.0436-25.2025</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Farran Briggs</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>['last_author', 'corresponding_author']</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>farran.briggs@nih.gov</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Translational Psychiatry</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>10.1038/s41398-025-03398-0</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Francesca McEwan</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>['first_author', 'corresponding_author']</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
+          <t>hackjinkim@korea.ac.kr</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>pattern</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactored the Paper class. Fixed the error of non-clean emails by decoding CloudFlare emails before cleaning them
</commit_message>
<xml_diff>
--- a/example_data/metadata.xlsx
+++ b/example_data/metadata.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,27 +473,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
+          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
+          <t>Psychedelic control of neuroimmune interactions governing fear</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1001-24.2025</t>
+          <t>10.1038/s41586-025-08880-9</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ekaterina Likhtik</t>
+          <t>Michael A. Wheeler</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>elikhtik@genectr.hunter.cuny.edu</t>
+          <t>mwheeler0@bwh.harvard.edu</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -515,37 +515,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03401-8</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Andreas Walther</t>
+          <t>Xinzhong Dong</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>a.walther@psychologie.uzh.ch</t>
+          <t>xdong2@jhmi.edu</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -557,37 +557,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tilman Stephani</t>
+          <t>Jun-Ming Zhang</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>tilman.stephani@donders.ru.nl</t>
+          <t>jun-ming.zhang@uc.edu</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -599,37 +599,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Vadim V. Nikulin</t>
+          <t>Ying Yu</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>nikulin@cbs.mpg.de</t>
+          <t>yuying@tmu.edu.cn</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -641,37 +641,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03322-6</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Ciyong Lu</t>
+          <t>Qiang Liu</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>luciyong@mail.sysu.edu.cn</t>
+          <t>qliu@tmu.edu.cn</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -683,37 +683,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2378-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Keise Izuma</t>
+          <t>Jie Zhou</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>izuma.keise@kochi-tech.ac.jp</t>
+          <t>zhoujie@tmu.edu.cn</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -725,37 +725,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1038/s41398-025-03398-0</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Xiaofen Zhong</t>
+          <t>Francesca McEwan</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>zhongxf29@mail.sysu.edu.cn</t>
+          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -777,27 +777,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1523/JNEUROSCI.1907-24.2025</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Weixiang Guo</t>
+          <t>Johanna B. Fritzinger</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>wxguo@genetics.ac.cn</t>
+          <t>johanna_fritzinger@URMC.rochester.edu</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -809,7 +809,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -819,17 +819,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
+          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2218-24.2025</t>
+          <t>10.1523/JNEUROSCI.0404-25.2025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bin He</t>
+          <t>Michael Vesia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>bhe1@andrew.cmu.edu</t>
+          <t>mvesia@umich.edu</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -851,37 +851,37 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1523/JNEUROSCI.1114-24.2025</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Xinzhong Dong</t>
+          <t>Hackjin Kim</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>xdong2@jhmi.edu</t>
+          <t>hackjinkim@korea.ac.kr</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -893,27 +893,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Jun-Ming Zhang</t>
+          <t>Gina G. Turrigiano</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>jun-ming.zhang@uc.edu</t>
+          <t>turrigiano@brandeis.edu</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -935,37 +935,37 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
+          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03393-5</t>
+          <t>10.1523/JNEUROSCI.0217-25.2025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Chi-Yung Shang</t>
+          <t>Shinya Ohara</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>cyshang@ntu.edu.tw</t>
+          <t>shinya.ohara.d3@tohoku.ac.jp</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -977,37 +977,37 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Grouping signals in primate visual cortex</t>
+          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.003</t>
+          <t>10.1523/JNEUROSCI.2187-24.2025</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Tom P. Franken</t>
+          <t>Min Wu</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>ftom@wustl.edu</t>
+          <t>min.wu@ndcn.ox.ac.uk</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1019,7 +1019,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1029,27 +1029,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
+          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2187-24.2025</t>
+          <t>10.1523/JNEUROSCI.0044-25.2025</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Min Wu</t>
+          <t>Bas Rokers</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>min.wu@ndcn.ox.ac.uk</t>
+          <t>rokers@nyu.edu</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1061,7 +1061,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1071,17 +1071,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Christoph Bamberg</t>
+          <t>Xiaodong Xu</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1091,19 +1091,19 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Christoph.bamberg@stud.plus.ac.at</t>
+          <t>412alix@gmail.com</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>proximity</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1113,143 +1113,143 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sarah Weigelt</t>
+          <t>Lijuan Chen</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>sarah.weigelt@tu-dortmund.de</t>
+          <t>clj0430@126.com</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>proximity</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1523/JNEUROSCI.1001-24.2025</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Xiaodong Xu</t>
+          <t>Ekaterina Likhtik</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>412alix@gmail.com</t>
+          <t>elikhtik@genectr.hunter.cuny.edu</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>proximity</t>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1038/s41398-025-03401-8</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Lijuan Chen</t>
+          <t>Andreas Walther</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>clj0430@126.com</t>
+          <t>a.walther@psychologie.uzh.ch</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>proximity</t>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
+          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
+          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0404-25.2025</t>
+          <t>10.1038/s41398-025-03390-8</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Michael Vesia</t>
+          <t>Ryan Smith</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>mvesia@umich.edu</t>
+          <t>rsmith@laureateinstitute.org</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1271,27 +1271,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Grouping signals in primate visual cortex</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1016/j.neuron.2025.05.003</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Karthik Srinivasan</t>
+          <t>Tom P. Franken</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>skarthik@mit.edu</t>
+          <t>ftom@wustl.edu</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1333,17 +1333,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Robert Desimone</t>
+          <t>Karthik Srinivasan</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>desimone@mit.edu</t>
+          <t>skarthik@mit.edu</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1355,37 +1355,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-24.2025</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Alapakkam P. Sampath</t>
+          <t>Robert Desimone</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>asampath@jsei.ucla.edu</t>
+          <t>desimone@mit.edu</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1397,37 +1397,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Lindsay A. Hohsfield</t>
+          <t>Xiaofen Zhong</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>lhohsfie@uci.edu</t>
+          <t>zhongxf29@mail.sysu.edu.cn</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1439,37 +1439,37 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Kim N. Green</t>
+          <t>Weixiang Guo</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>kngreen@uci.edu</t>
+          <t>wxguo@genetics.ac.cn</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1481,37 +1481,37 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
+          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1876-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.018</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Lidon Marin-Marin</t>
+          <t>Qingtao Sun</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>lidon.marinmarin@york.ac.uk</t>
+          <t>qsun@cshl.edu</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1523,37 +1523,37 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2418176122</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Megan M. Davis</t>
+          <t>Amy Hauck Newman</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>davismeg@unc.edu</t>
+          <t>anewman@intra.nida.nih.gov</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1565,37 +1565,37 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2411669122</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Olivier Thoumine</t>
+          <t>Zheng-Xiong Xi</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>olivier.thoumine@u-bordeaux.fr</t>
+          <t>zxi@intra.nida.nih.gov</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1617,27 +1617,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1788-24.2025</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Mingzhou Ding</t>
+          <t>Tilman Stephani</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>mding@bme.ufl.edu</t>
+          <t>tilman.stephani@donders.ru.nl</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1649,7 +1649,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1659,17 +1659,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0044-25.2025</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Bas Rokers</t>
+          <t>Vadim V. Nikulin</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>rokers@nyu.edu</t>
+          <t>nikulin@cbs.mpg.de</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1691,37 +1691,37 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Psychedelic control of neuroimmune interactions governing fear</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08880-9</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Michael A. Wheeler</t>
+          <t>Wenjie Zhou</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>mwheeler0@bwh.harvard.edu</t>
+          <t>zhouwj2022@shsmu.edu.cn</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1733,37 +1733,37 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2186-24.2025</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Siyi Chen (陈思佚)</t>
+          <t>Wenxi Huang</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Siyi.Chen@psy.lmu.de</t>
+          <t>tw.huang@siat.ac.cn</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1775,37 +1775,37 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0217-25.2025</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Shinya Ohara</t>
+          <t>Yuanyuan Liu</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>shinya.ohara.d3@tohoku.ac.jp</t>
+          <t>yuanyuan.liu@nih.gov</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1817,37 +1817,37 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1038/s41398-025-03392-6</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Stuart Berg</t>
+          <t>Christelle Langley</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>bergs@janelia.hhmi.org</t>
+          <t>cl798@medschl.cam.ac.uk</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1859,37 +1859,37 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1523/JNEUROSCI.0491-25.2025</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Gerald M. Rubin</t>
+          <t>Barry J. Richmond</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>rubing@janelia.hhmi.org</t>
+          <t>barryrichmond@mail.nih.gov</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1901,37 +1901,37 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1523/JNEUROSCI.2186-24.2025</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Michael B. Reiser</t>
+          <t>Siyi Chen (陈思佚)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>reiserm@janelia.hhmi.org</t>
+          <t>Siyi.Chen@psy.lmu.de</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1943,37 +1943,37 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Ying Yu</t>
+          <t>Yulong Li</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>yuying@tmu.edu.cn</t>
+          <t>yulongli@pku.edu.cn</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1985,37 +1985,37 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1038/s41398-025-03322-6</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Qiang Liu</t>
+          <t>Ciyong Lu</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>qliu@tmu.edu.cn</t>
+          <t>luciyong@mail.sysu.edu.cn</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2027,37 +2027,37 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.1920-23.2025</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Jie Zhou</t>
+          <t>Adrianna C. Jenkins</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>zhoujie@tmu.edu.cn</t>
+          <t>acjenk@upenn.edu</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2069,7 +2069,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2079,27 +2079,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1523/JNEUROSCI.2378-24.2025</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Yan Chen</t>
+          <t>Keise Izuma</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>chen_yan@hznu.edu.cn</t>
+          <t>izuma.keise@kochi-tech.ac.jp</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2111,7 +2111,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2121,17 +2121,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1523/JNEUROSCI.2218-24.2025</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Haibo Di</t>
+          <t>Bin He</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>haibodi@hznu.edu.cn</t>
+          <t>bhe1@andrew.cmu.edu</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2153,27 +2153,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>A neural basis for distinguishing imagination from reality</t>
+          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.015</t>
+          <t>10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Nadine Dijkstra</t>
+          <t>Megan M. Davis</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>n.dijkstra@ucl.ac.uk</t>
+          <t>davismeg@unc.edu</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2195,7 +2195,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2205,27 +2205,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Activity-dependent development of the body’s touch receptors</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.04.015</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>David D. Ginty</t>
+          <t>Adam P. Caccavano</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>david_ginty@hms.harvard.edu</t>
+          <t>adam.caccavano@nih.gov</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2237,37 +2237,37 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1139-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Paula T. Kuokkanen</t>
+          <t>Kenneth A. Pelkey</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>paula.kuokkanen@hu-berlin.de</t>
+          <t>pelkeyk2@mail.nih.gov</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2279,37 +2279,37 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Shigehiro Ohdo</t>
+          <t>Chris J. McBain</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>ohdo@phar.kyushu-u.ac.jp</t>
+          <t>mcbainc@mail.nih.gov</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2321,7 +2321,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2331,17 +2331,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1523/JNEUROSCI.0436-25.2025</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Satoru Koyanagi</t>
+          <t>Farran Briggs</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>koyanagi@phar.kyushu-u.ac.jp</t>
+          <t>farran.briggs@nih.gov</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2363,7 +2363,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2373,27 +2373,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Cong Liu</t>
+          <t>Lindsay A. Hohsfield</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>liulab@sioc.ac.cn</t>
+          <t>lhohsfie@uci.edu</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2405,7 +2405,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2415,27 +2415,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ShengQi Xiang</t>
+          <t>Kim N. Green</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>cqxiang@ustc.edu.cn</t>
+          <t>kngreen@uci.edu</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2457,27 +2457,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.019</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Zhuohao He</t>
+          <t>Wang Zheng</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>hezh@sioc.ac.cn</t>
+          <t>wzheng86@wisc.edu</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2489,27 +2489,27 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2504775122</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Gina G. Turrigiano</t>
+          <t>Jeffrey R. Holt</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>turrigiano@brandeis.edu</t>
+          <t>jeffrey.holt@childrens.harvard.edu</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2531,7 +2531,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2541,27 +2541,27 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Jae-Chang Kim</t>
+          <t>Jocelyn M. Breton</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>jaechang.kim@econ.uzh.ch</t>
+          <t>jo.breton@northeastern.edu</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2573,7 +2573,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Philippe N. Tobler</t>
+          <t>Inbal Ben-Ami Bartal</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>phil.tobler@econ.uzh.ch</t>
+          <t>inbalbe@tauex.tau.ac.il</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2615,27 +2615,27 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1907-24.2025</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Johanna B. Fritzinger</t>
+          <t>Christoph Bamberg</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>johanna_fritzinger@URMC.rochester.edu</t>
+          <t>Christoph.bamberg@stud.plus.ac.at</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2657,37 +2657,37 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2325-24.2025</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Martha E. Bickford</t>
+          <t>Sarah Weigelt</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>martha.bickford@louisville.edu</t>
+          <t>sarah.weigelt@tu-dortmund.de</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2699,37 +2699,37 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Jocelyn M. Breton</t>
+          <t>Olivier Thoumine</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>jo.breton@northeastern.edu</t>
+          <t>olivier.thoumine@u-bordeaux.fr</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2741,37 +2741,37 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>A neural basis for distinguishing imagination from reality</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.015</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Inbal Ben-Ami Bartal</t>
+          <t>Nadine Dijkstra</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>inbalbe@tauex.tau.ac.il</t>
+          <t>n.dijkstra@ucl.ac.uk</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2783,37 +2783,37 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.018</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Qingtao Sun</t>
+          <t>Takahiro Morito</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>qsun@cshl.edu</t>
+          <t>takahiro.morito@riken.jp</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2835,17 +2835,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-23.2025</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Adrianna C. Jenkins</t>
+          <t>Takaomi C. Saido</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2855,7 +2855,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>acjenk@upenn.edu</t>
+          <t>takaomi.saido@riken.jp</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2867,37 +2867,37 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03399-z</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Cristina Benatti</t>
+          <t>Cephra Raja</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>cristina.benatti@unimore.it</t>
+          <t>cr2163@stanford.edu</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2909,37 +2909,37 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03392-6</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Christelle Langley</t>
+          <t>Vivek Buch</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>cl798@medschl.cam.ac.uk</t>
+          <t>vpbuch@stanford.edu</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2951,37 +2951,37 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0491-25.2025</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Barry J. Richmond</t>
+          <t>Karl Deisseroth</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>barryrichmond@mail.nih.gov</t>
+          <t>deissero@stanford.edu</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2993,37 +2993,37 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1523/JNEUROSCI.2325-24.2025</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Amy Hauck Newman</t>
+          <t>Martha E. Bickford</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>anewman@intra.nida.nih.gov</t>
+          <t>martha.bickford@louisville.edu</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3035,37 +3035,37 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Zheng-Xiong Xi</t>
+          <t>Shigehiro Ohdo</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>zxi@intra.nida.nih.gov</t>
+          <t>ohdo@phar.kyushu-u.ac.jp</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3077,27 +3077,27 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03390-8</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Ryan Smith</t>
+          <t>Satoru Koyanagi</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>rsmith@laureateinstitute.org</t>
+          <t>koyanagi@phar.kyushu-u.ac.jp</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3119,37 +3119,37 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1038/s41398-025-03399-z</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Ethan B. Richman</t>
+          <t>Cristina Benatti</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>deissero@stanford.edu</t>
+          <t>cristina.benatti@unimore.it</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3161,37 +3161,37 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Cephra Raja</t>
+          <t>Jae-Chang Kim</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>cr2163@stanford.edu</t>
+          <t>jaechang.kim@econ.uzh.ch</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3203,37 +3203,37 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Vivek Buch</t>
+          <t>Philippe N. Tobler</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>vpbuch@stanford.edu</t>
+          <t>phil.tobler@econ.uzh.ch</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3245,37 +3245,37 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.jneurosci.org/content/45/22/e1920242025</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>The Role of the Ca&lt;sup&gt;2+&lt;/sup&gt;-activated Cl&lt;sup&gt;−&lt;/sup&gt;Conductance in the Membrane Potential and Light Response of Mouse Rods</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1523/JNEUROSCI.1920-24.2025</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Karl Deisseroth</t>
+          <t>Alapakkam P. Sampath</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>deissero@stanford.edu?cc=vpbuch@stanford.edu&amp;amp;cc=cr2163@stanford.edu&amp;amp;cc=23sciencemag@pn.stanford.edu</t>
+          <t>asampath@jsei.ucla.edu</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3287,27 +3287,27 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03398-0</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Francesca McEwan</t>
+          <t>Adam Steel</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
+          <t>adamdanielsteel@gmail.com</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3329,27 +3329,27 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03272-z</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Froukje E. de Vries</t>
+          <t>Caroline E. Robertson</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3359,19 +3359,19 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>f.d.vries@nki.nl</t>
+          <t>cerw@dartmouth.edu</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>pattern</t>
+          <t>proximity</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3381,27 +3381,27 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
+          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0436-25.2025</t>
+          <t>10.1523/JNEUROSCI.1139-24.2025</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Farran Briggs</t>
+          <t>Paula T. Kuokkanen</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>farran.briggs@nih.gov</t>
+          <t>paula.kuokkanen@hu-berlin.de</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3413,37 +3413,37 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.1788-24.2025</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Adam P. Caccavano</t>
+          <t>Mingzhou Ding</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>adam.caccavano@nih.gov</t>
+          <t>mding@bme.ufl.edu</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3455,37 +3455,37 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.1876-24.2025</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Kenneth A. Pelkey</t>
+          <t>Lidon Marin-Marin</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>pelkeyk2@mail.nih.gov</t>
+          <t>lidon.marinmarin@york.ac.uk</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3497,37 +3497,37 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1038/s41398-025-03393-5</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Chris J. McBain</t>
+          <t>Chi-Yung Shang</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>mcbainc@mail.nih.gov</t>
+          <t>cyshang@ntu.edu.tw</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3539,7 +3539,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3549,27 +3549,27 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Wang Zheng</t>
+          <t>Cong Liu</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>wzheng86@wisc.edu</t>
+          <t>liulab@sioc.ac.cn</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3581,7 +3581,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3591,27 +3591,27 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Jeffrey R. Holt</t>
+          <t>ShengQi Xiang</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>jeffrey.holt@childrens.harvard.edu</t>
+          <t>cqxiang@ustc.edu.cn</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3623,27 +3623,27 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00219-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
+          <t>Fibril fuzzy coat is important for α-synuclein pathological transmission activity</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>10.1126/science.adt7705</t>
+          <t>10.1016/j.neuron.2025.03.019</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Yulong Li</t>
+          <t>Zhuohao He</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>yulongli@pku.edu.cn</t>
+          <t>hezh@sioc.ac.cn</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3665,37 +3665,37 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Activity-dependent development of the body’s touch receptors</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1016/j.neuron.2025.04.015</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Marie-Lucie Read</t>
+          <t>David D. Ginty</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>readms2@cardiff.ac.uk</t>
+          <t>david_ginty@hms.harvard.edu</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3707,37 +3707,37 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1038/s41398-025-03272-z</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Andrew D. Lawrence</t>
+          <t>Froukje E. de Vries</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Andrew.D.Lawrence@ed.ac.uk</t>
+          <t>f.d.vries@nki.nl</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3749,7 +3749,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3759,17 +3759,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Adam Steel</t>
+          <t>Marie-Lucie Read</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>adamdanielsteel@gmail.com</t>
+          <t>readms2@cardiff.ac.uk</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3791,7 +3791,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3801,39 +3801,39 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Caroline E. Robertson</t>
+          <t>Andrew D. Lawrence</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>cerw@dartmouth.edu</t>
+          <t>Andrew.D.Lawrence@ed.ac.uk</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>proximity</t>
+          <t>pattern</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3843,17 +3843,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Takahiro Morito</t>
+          <t>Yan Chen</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>takahiro.morito@riken.jp</t>
+          <t>chen_yan@hznu.edu.cn</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3875,7 +3875,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3885,17 +3885,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Takaomi C. Saido</t>
+          <t>Haibo Di</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>takaomi.saido@riken.jp</t>
+          <t>haibodi@hznu.edu.cn</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3917,40 +3917,124 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1114-24.2025</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Hackjin Kim</t>
+          <t>Stuart Berg</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
+          <t>['corresponding_author']</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>bergs@janelia.hhmi.org</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>10.1038/s41586-025-08746-0</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Gerald M. Rubin</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>['corresponding_author']</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>rubing@janelia.hhmi.org</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>10.1038/s41586-025-08746-0</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Michael B. Reiser</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
           <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>hackjinkim@korea.ac.kr</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr">
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>reiserm@janelia.hhmi.org</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>

</xml_diff>

<commit_message>
Added a flag to indicate when there is an ambiguous match that must be sorted manually.
</commit_message>
<xml_diff>
--- a/example_data/metadata.xlsx
+++ b/example_data/metadata.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,53 +469,61 @@
           <t>match_method</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ambiguous</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Psychedelic control of neuroimmune interactions governing fear</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08880-9</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Michael A. Wheeler</t>
+          <t>Wang Zheng</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>mwheeler0@bwh.harvard.edu</t>
+          <t>wzheng86@wisc.edu</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -525,249 +533,267 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1016/j.neuron.2025.05.009</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Xinzhong Dong</t>
+          <t>Jeffrey R. Holt</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>xdong2@jhmi.edu</t>
+          <t>jeffrey.holt@childrens.harvard.edu</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
+          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.006</t>
+          <t>10.1523/JNEUROSCI.1788-24.2025</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Jun-Ming Zhang</t>
+          <t>Mingzhou Ding</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>jun-ming.zhang@uc.edu</t>
+          <t>mding@bme.ufl.edu</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ying Yu</t>
+          <t>Xiaofen Zhong</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>yuying@tmu.edu.cn</t>
+          <t>zhongxf29@mail.sysu.edu.cn</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.0370-25.2025</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Qiang Liu</t>
+          <t>Weixiang Guo</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>qliu@tmu.edu.cn</t>
+          <t>wxguo@genetics.ac.cn</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.014</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Jie Zhou</t>
+          <t>Jocelyn M. Breton</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>zhoujie@tmu.edu.cn</t>
+          <t>jo.breton@northeastern.edu</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
+          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03398-0</t>
+          <t>10.1523/JNEUROSCI.0845-24.2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Francesca McEwan</t>
+          <t>Inbal Ben-Ami Bartal</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
+          <t>inbalbe@tauex.tau.ac.il</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -777,39 +803,42 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
+          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1907-24.2025</t>
+          <t>10.1523/JNEUROSCI.2378-24.2025</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Johanna B. Fritzinger</t>
+          <t>Keise Izuma</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>johanna_fritzinger@URMC.rochester.edu</t>
+          <t>izuma.keise@kochi-tech.ac.jp</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I9" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -819,17 +848,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
+          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0404-25.2025</t>
+          <t>10.1523/JNEUROSCI.1114-24.2025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Michael Vesia</t>
+          <t>Hackjin Kim</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -839,19 +868,22 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>mvesia@umich.edu</t>
+          <t>hackjinkim@korea.ac.kr</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1114242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -861,375 +893,402 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Neural Processes Linking Interoception to Moral Preferences Aligned with Group Consensus</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1114-24.2025</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hackjin Kim</t>
+          <t>Takahiro Morito</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>hackjinkim@korea.ac.kr</t>
+          <t>takahiro.morito@riken.jp</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
+          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
+          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2504775122</t>
+          <t>10.1523/JNEUROSCI.2152-24.2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Gina G. Turrigiano</t>
+          <t>Takaomi C. Saido</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>turrigiano@brandeis.edu</t>
+          <t>takaomi.saido@riken.jp</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0217-25.2025</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Shinya Ohara</t>
+          <t>Xinzhong Dong</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>shinya.ohara.d3@tohoku.ac.jp</t>
+          <t>xdong2@jhmi.edu</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I13" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00178-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
+          <t>Vascular motion in the dorsal root ganglion sensed by Piezo2 in sensory neurons triggers episodic pain</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2187-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.006</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Min Wu</t>
+          <t>Jun-Ming Zhang</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>min.wu@ndcn.ox.ac.uk</t>
+          <t>jun-ming.zhang@uc.edu</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0044-25.2025</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Bas Rokers</t>
+          <t>Lindsay A. Hohsfield</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>rokers@nyu.edu</t>
+          <t>lhohsfie@uci.edu</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I15" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1016/j.neuron.2025.05.004</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Xiaodong Xu</t>
+          <t>Kim N. Green</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>412alix@gmail.com</t>
+          <t>kngreen@uci.edu</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>proximity</t>
-        </is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="I16" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
+          <t>Modular arrangement of synaptic and intrinsic homeostatic plasticity within visual cortical circuits</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00327-0</t>
+          <t>10.1073/pnas.2504775122</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Lijuan Chen</t>
+          <t>Gina G. Turrigiano</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>clj0430@126.com</t>
+          <t>turrigiano@brandeis.edu</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>proximity</t>
-        </is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="I17" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
+          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1001-24.2025</t>
+          <t>10.1038/s41398-025-03392-6</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ekaterina Likhtik</t>
+          <t>Christelle Langley</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>elikhtik@genectr.hunter.cuny.edu</t>
+          <t>cl798@medschl.cam.ac.uk</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
+          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03401-8</t>
+          <t>10.1523/JNEUROSCI.0491-25.2025</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Andreas Walther</t>
+          <t>Barry J. Richmond</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>a.walther@psychologie.uzh.ch</t>
+          <t>barryrichmond@mail.nih.gov</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I19" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1239,165 +1298,177 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03390-8</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ryan Smith</t>
+          <t>Amy Hauck Newman</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>rsmith@laureateinstitute.org</t>
+          <t>anewman@intra.nida.nih.gov</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I20" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Grouping signals in primate visual cortex</t>
+          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.003</t>
+          <t>10.1038/s41398-025-03391-7</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tom P. Franken</t>
+          <t>Zheng-Xiong Xi</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>ftom@wustl.edu</t>
+          <t>zxi@intra.nida.nih.gov</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I21" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Karthik Srinivasan</t>
+          <t>Christoph Bamberg</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>skarthik@mit.edu</t>
+          <t>Christoph.bamberg@stud.plus.ac.at</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I22" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
+          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
+          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2420704122</t>
+          <t>10.1038/s41539-025-00308-3</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Robert Desimone</t>
+          <t>Sarah Weigelt</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>desimone@mit.edu</t>
+          <t>sarah.weigelt@tu-dortmund.de</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I23" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1407,39 +1478,42 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Xiaofen Zhong</t>
+          <t>Tilman Stephani</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>zhongxf29@mail.sysu.edu.cn</t>
+          <t>tilman.stephani@donders.ru.nl</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I24" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0370252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1449,17 +1523,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Targeting Lysine α-Ketoglutarate Reductase to Treat Pyridoxine-Dependent Epilepsy</t>
+          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0370-25.2025</t>
+          <t>10.1523/JNEUROSCI.2280-24.2025</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Weixiang Guo</t>
+          <t>Vadim V. Nikulin</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1469,103 +1543,112 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>wxguo@genetics.ac.cn</t>
+          <t>nikulin@cbs.mpg.de</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I25" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e0044252025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
+          <t>Single-Trial fMRI Decoding of 3D Motion with Stereoscopic and Perspective Cues</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.018</t>
+          <t>10.1523/JNEUROSCI.0044-25.2025</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Qingtao Sun</t>
+          <t>Bas Rokers</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>qsun@cshl.edu</t>
+          <t>rokers@nyu.edu</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I26" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Activity-dependent development of the body’s touch receptors</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1016/j.neuron.2025.04.015</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Amy Hauck Newman</t>
+          <t>David D. Ginty</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>anewman@intra.nida.nih.gov</t>
+          <t>david_ginty@hms.harvard.edu</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I27" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03391-7?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03401-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1575,81 +1658,87 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>RDS-04-010: a novel atypical DAT inhibitor that inhibits cocaine taking and seeking and itself has low abuse potential in experimental animals</t>
+          <t>Major depressive disorder in children and adolescents is associated with reduced hair cortisol and anandamide (AEA): cross-sectional and longitudinal evidence from a large randomized clinical trial</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03391-7</t>
+          <t>10.1038/s41398-025-03401-8</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Zheng-Xiong Xi</t>
+          <t>Andreas Walther</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>zxi@intra.nida.nih.gov</t>
+          <t>a.walther@psychologie.uzh.ch</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I28" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1038/s41398-025-03399-z</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Tilman Stephani</t>
+          <t>Cristina Benatti</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>tilman.stephani@donders.ru.nl</t>
+          <t>cristina.benatti@unimore.it</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I29" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2280242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e2187242025</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1659,39 +1748,42 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Excitability Modulations of Somatosensory Perception Do Not Depend on Feedforward Neuronal Population Spikes</t>
+          <t>Differential Beta and Gamma Activity Modulation during Unimanual and Bimanual Motor Learning</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2280-24.2025</t>
+          <t>10.1523/JNEUROSCI.2187-24.2025</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Vadim V. Nikulin</t>
+          <t>Min Wu</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nikulin@cbs.mpg.de</t>
+          <t>min.wu@ndcn.ox.ac.uk</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I30" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00350-2?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1701,101 +1793,107 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Grouping signals in primate visual cortex</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1016/j.neuron.2025.05.003</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Wenjie Zhou</t>
+          <t>Tom P. Franken</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>zhouwj2022@shsmu.edu.cn</t>
+          <t>ftom@wustl.edu</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I31" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Wenxi Huang</t>
+          <t>Karthik Srinivasan</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>tw.huang@siat.ac.cn</t>
+          <t>skarthik@mit.edu</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I32" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>A pontine center in descending pain control</t>
+          <t>Stimulus representations in visual cortex shaped by spatial attention and microsaccades</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.02.028</t>
+          <t>10.1073/pnas.2420704122</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Yuanyuan Liu</t>
+          <t>Robert Desimone</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1805,19 +1903,22 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>yuanyuan.liu@nih.gov</t>
+          <t>desimone@mit.edu</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I33" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03392-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1827,39 +1928,42 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Computational modelling and neural correlates of reinforcement learning following three-week escitalopram: a double-blind, placebo-controlled semi-randomised study</t>
+          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03392-6</t>
+          <t>10.1038/s41398-025-03322-6</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Christelle Langley</t>
+          <t>Ciyong Lu</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>cl798@medschl.cam.ac.uk</t>
+          <t>luciyong@mail.sysu.edu.cn</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I34" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0491252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1001242025</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1869,17 +1973,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Chemogenetic Disruption of Monkey Perirhinal Neurons Projecting to the Rostromedial Caudate Impairs Associative Learning</t>
+          <t>Infralimbic Projections to the Substantia Innominata–Ventral Pallidum Constrain Defensive Behavior during Extinction Learning</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0491-25.2025</t>
+          <t>10.1523/JNEUROSCI.1001-24.2025</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Barry J. Richmond</t>
+          <t>Ekaterina Likhtik</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1889,39 +1993,42 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>barryrichmond@mail.nih.gov</t>
+          <t>elikhtik@genectr.hunter.cuny.edu</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I35" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
+          <t>A neural basis for distinguishing imagination from reality</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2186-24.2025</t>
+          <t>10.1016/j.neuron.2025.05.015</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Siyi Chen (陈思佚)</t>
+          <t>Nadine Dijkstra</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1931,103 +2038,112 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Siyi.Chen@psy.lmu.de</t>
+          <t>n.dijkstra@ucl.ac.uk</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I36" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
+          <t>https://www.jneurosci.org/content/45/22/e2186242025</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
+          <t>Statistical Context Learning in Visual Search: Distinct Electrophysiological Signatures of Contextual Guidance and Context Suppression</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10.1126/science.adt7705</t>
+          <t>10.1523/JNEUROSCI.2186-24.2025</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Yulong Li</t>
+          <t>Siyi Chen (陈思佚)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>yulongli@pku.edu.cn</t>
+          <t>Siyi.Chen@psy.lmu.de</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I37" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03322-6?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Perceived criticism and depressive symptoms among adults aged 50 years and older: a 17-year population-based cohort study</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03322-6</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Ciyong Lu</t>
+          <t>Shigehiro Ohdo</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>luciyong@mail.sysu.edu.cn</t>
+          <t>ohdo@phar.kyushu-u.ac.jp</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I38" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2037,17 +2153,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
+          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1920-23.2025</t>
+          <t>10.1523/JNEUROSCI.1969-24.2025</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Adrianna C. Jenkins</t>
+          <t>Satoru Koyanagi</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2057,249 +2173,267 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>acjenk@upenn.edu</t>
+          <t>koyanagi@phar.kyushu-u.ac.jp</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I39" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2378242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Decomposing Cognitive Processes in the mPFC during Self-Thinking</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2378-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Keise Izuma</t>
+          <t>Ying Yu</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>izuma.keise@kochi-tech.ac.jp</t>
+          <t>yuying@tmu.edu.cn</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I40" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2218-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Bin He</t>
+          <t>Qiang Liu</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>bhe1@andrew.cmu.edu</t>
+          <t>qliu@tmu.edu.cn</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I41" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00186-2?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
+          <t>ILC2 instructs neural stem and progenitor cells to potentiate neurorepair after stroke</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2418176122</t>
+          <t>10.1016/j.neuron.2025.03.014</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Megan M. Davis</t>
+          <t>Jie Zhou</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>davismeg@unc.edu</t>
+          <t>zhoujie@tmu.edu.cn</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I42" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.0436-25.2025</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Adam P. Caccavano</t>
+          <t>Farran Briggs</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>adam.caccavano@nih.gov</t>
+          <t>farran.briggs@nih.gov</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I43" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e1907242025</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>Mechanisms of Tone-in-Noise Encoding in the Inferior Colliculus</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.1907-24.2025</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Kenneth A. Pelkey</t>
+          <t>Johanna B. Fritzinger</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>pelkeyk2@mail.nih.gov</t>
+          <t>johanna_fritzinger@URMC.rochester.edu</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I44" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
+          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.03.005</t>
+          <t>10.1523/JNEUROSCI.2325-24.2025</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Chris J. McBain</t>
+          <t>Martha E. Bickford</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2309,19 +2443,22 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>mcbainc@mail.nih.gov</t>
+          <t>martha.bickford@louisville.edu</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I45" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0436252025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2331,123 +2468,132 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Differential Impact of Retinal Lesions on Visual Responses of LGN X and Y Cells</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0436-25.2025</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Farran Briggs</t>
+          <t>Yan Chen</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>farran.briggs@nih.gov</t>
+          <t>chen_yan@hznu.edu.cn</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I46" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1523/JNEUROSCI.1684-24.2025</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Lindsay A. Hohsfield</t>
+          <t>Haibo Di</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>lhohsfie@uci.edu</t>
+          <t>haibodi@hznu.edu.cn</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I47" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00351-4?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Identification of the velum interpositum as a meningeal-CNS route for myeloid cell trafficking into the brain</t>
+          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.004</t>
+          <t>10.1523/JNEUROSCI.1139-24.2025</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Kim N. Green</t>
+          <t>Paula T. Kuokkanen</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>kngreen@uci.edu</t>
+          <t>paula.kuokkanen@hu-berlin.de</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I48" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00218-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2457,17 +2603,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>Dynorphin modulates reward-seeking actions through a pallido-amygdala cholinergic circuit</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1016/j.neuron.2025.03.018</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Wang Zheng</t>
+          <t>Qingtao Sun</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2477,249 +2623,267 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>wzheng86@wisc.edu</t>
+          <t>qsun@cshl.edu</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I49" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00356-3?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Structural and functional basis of mechanosensitive TMEM63 channelopathies</t>
+          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.009</t>
+          <t>10.1523/JNEUROSCI.1876-24.2025</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Jeffrey R. Holt</t>
+          <t>Lidon Marin-Marin</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>jeffrey.holt@childrens.harvard.edu</t>
+          <t>lidon.marinmarin@york.ac.uk</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I50" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Jocelyn M. Breton</t>
+          <t>Eun Young Choi</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>jo.breton@northeastern.edu</t>
+          <t>23sciencemag@pn.stanford.edu</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I51" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e0845242025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Neural and Behavioral Correlates of Individual Variability in Rat Helping Behavior: A Role for Social Affiliation and Oxytocin Receptors</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0845-24.2025</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Inbal Ben-Ami Bartal</t>
+          <t>Cephra Raja</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>inbalbe@tauex.tau.ac.il</t>
+          <t>cr2163@stanford.edu</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I52" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Christoph Bamberg</t>
+          <t>Carolyn I. Rodríguez</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Christoph.bamberg@stud.plus.ac.at</t>
+          <t>cr2163@stanford.edu</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I53" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41539-025-00308-3?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>npj Science of Learning</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Reversal learning is influenced by cognitive flexibility and develops throughout early adolescence</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10.1038/s41539-025-00308-3</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Sarah Weigelt</t>
+          <t>Vivek Buch</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>sarah.weigelt@tu-dortmund.de</t>
+          <t>vpbuch@stanford.edu</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I54" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
+          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Proceedings of the National Academy of Sciences</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
+          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>10.1073/pnas.2411669122</t>
+          <t>10.1126/science.adt3971</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Olivier Thoumine</t>
+          <t>Karl Deisseroth</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2729,61 +2893,67 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>olivier.thoumine@u-bordeaux.fr</t>
+          <t>deissero@stanford.edu</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I55" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00362-9?dgcid=raven_jbs_aip_email</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>A neural basis for distinguishing imagination from reality</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.05.015</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Nadine Dijkstra</t>
+          <t>Marie-Lucie Read</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>['first_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>n.dijkstra@ucl.ac.uk</t>
+          <t>readms2@cardiff.ac.uk</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I56" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2793,101 +2963,107 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1523/JNEUROSCI.1700-24.2025</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Takahiro Morito</t>
+          <t>Andrew D. Lawrence</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>takahiro.morito@riken.jp</t>
+          <t>Andrew.D.Lawrence@ed.ac.uk</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I57" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2152242025</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>The Role of Neprilysin and Insulin-Degrading Enzyme in the Etiology of Sporadic Alzheimer's Disease</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2152-24.2025</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Takaomi C. Saido</t>
+          <t>Xiaodong Xu</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>takaomi.saido@riken.jp</t>
+          <t>412alix@gmail.com</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I58" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.nature.com/articles/s41539-025-00327-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41539_AWA1_GL_DTEC_054CI_TOC-250528&amp;utm_content=20250528</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>npj Science of Learning</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Unveiling the neural mechanisms of supernatural fiction comprehension using fNIRS</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1038/s41539-025-00327-0</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Cephra Raja</t>
+          <t>Cheng Jia</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2897,165 +3073,177 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>cr2163@stanford.edu</t>
+          <t>clj0430@126.com</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I59" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1038/s41398-025-03272-z</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Vivek Buch</t>
+          <t>Froukje E. de Vries</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>vpbuch@stanford.edu</t>
+          <t>f.d.vries@nki.nl</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I60" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.science.org/doi/10.1126/science.adt3971</t>
+          <t>https://www.jneurosci.org/content/45/23/e2218242025</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Conserved brain-wide emergence of emotional response from sensory experience in humans and mice</t>
+          <t>Transcranial Focused Ultrasound Modulates Feedforward and Feedback Cortico-Thalamo-Cortical Pathways by Selectively Activating Excitatory Neurons</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>10.1126/science.adt3971</t>
+          <t>10.1523/JNEUROSCI.2218-24.2025</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Karl Deisseroth</t>
+          <t>Bin He</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>deissero@stanford.edu</t>
+          <t>bhe1@andrew.cmu.edu</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I61" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e2325242025</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>GABAergic Projections from the Pretectum Boost Retinogeniculate Signal Transfer via Disinhibition</t>
+          <t>Longitudinal associations between birth-to-six cortical growth and childhood neurocognitive function</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2325-24.2025</t>
+          <t>10.1073/pnas.2418176122</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Martha E. Bickford</t>
+          <t>Megan M. Davis</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>martha.bickford@louisville.edu</t>
+          <t>davismeg@unc.edu</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I62" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1038/s41398-025-03393-5</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Shigehiro Ohdo</t>
+          <t>Chi-Yung Shang</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -3065,181 +3253,196 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>ohdo@phar.kyushu-u.ac.jp</t>
+          <t>cyshang@ntu.edu.tw</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I63" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1969242025</t>
+          <t>https://www.science.org/doi/10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>The Circadian Clock Component REV-ERB Is an Analgesic Target for Cancer-Induced Tactile Pain Hypersensitivity</t>
+          <t>In vivo multiplex imaging of dynamic neurochemical networks with designed far-red dopamine sensors</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1969-24.2025</t>
+          <t>10.1126/science.adt7705</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Satoru Koyanagi</t>
+          <t>Yulong Li</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>koyanagi@phar.kyushu-u.ac.jp</t>
+          <t>yulongli@pku.edu.cn</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I64" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03399-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>First evidence of an anxiety-like behavior and its pharmacological modulation in a molluscan model organism, Lymnaea stagnalis</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03399-z</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Cristina Benatti</t>
+          <t>Adam P. Caccavano</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author']</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>cristina.benatti@unimore.it</t>
+          <t>adam.caccavano@nih.gov</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I65" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Jae-Chang Kim</t>
+          <t>Kenneth A. Pelkey</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>jaechang.kim@econ.uzh.ch</t>
+          <t>pelkeyk2@mail.nih.gov</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I66" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00177-1?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
+          <t>Divergent opioid-mediated suppression of inhibition between hippocampus and neocortex across species and development</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.2302-24.2025</t>
+          <t>10.1016/j.neuron.2025.03.005</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Philippe N. Tobler</t>
+          <t>Chris J. McBain</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>phil.tobler@econ.uzh.ch</t>
+          <t>mcbainc@mail.nih.gov</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I67" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -3283,11 +3486,14 @@
           <t>pattern</t>
         </is>
       </c>
+      <c r="I68" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.jneurosci.org/content/45/23/e0404252025</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3297,123 +3503,132 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Cerebellar Activity Affects Distal Cortical Physiology and Synaptic Plasticity in a Human Parietal–Motor Pathway Associated with Motor Actions</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1523/JNEUROSCI.0404-25.2025</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Adam Steel</t>
+          <t>Michael Vesia</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>adamdanielsteel@gmail.com</t>
+          <t>mvesia@umich.edu</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I69" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
+          <t>https://www.nature.com/articles/s41398-025-03398-0?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
+          <t>Association between redox dysregulation and vulnerability to cognitive deficits induced by maternal immune activation</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.0028-25.2025</t>
+          <t>10.1038/s41398-025-03398-0</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Caroline E. Robertson</t>
+          <t>Francesca McEwan</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>cerw@dartmouth.edu</t>
+          <t>francesca.mcewan@postgrad.manchester.ac.uk</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>proximity</t>
-        </is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="I70" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1139242025</t>
+          <t>https://www.nature.com/articles/s41586-025-08880-9?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Single Neuron Contributions to the Auditory Brainstem EEG</t>
+          <t>Psychedelic control of neuroimmune interactions governing fear</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1139-24.2025</t>
+          <t>10.1038/s41586-025-08880-9</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Paula T. Kuokkanen</t>
+          <t>Michael A. Wheeler</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>paula.kuokkanen@hu-berlin.de</t>
+          <t>mwheeler0@bwh.harvard.edu</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I71" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/23/e1788242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3423,39 +3638,42 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Stimulus Repetition Induces a Two-Stage Learning Process in the Primary Visual Cortex</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1788-24.2025</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Mingzhou Ding</t>
+          <t>Jae-Chang Kim</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>mding@bme.ufl.edu</t>
+          <t>jaechang.kim@econ.uzh.ch</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I72" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1876242025</t>
+          <t>https://www.jneurosci.org/content/45/23/e2302242025</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3465,75 +3683,81 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Whole-Brain Dimensions of Intrinsic Connectivity Capture Modality-Specific and Heteromodal Language Representations</t>
+          <t>The Anterior Insula Processes a Time-Resolved Subjective Risk Prediction Error</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1876-24.2025</t>
+          <t>10.1523/JNEUROSCI.2302-24.2025</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Lidon Marin-Marin</t>
+          <t>Philippe N. Tobler</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>lidon.marinmarin@york.ac.uk</t>
+          <t>phil.tobler@econ.uzh.ch</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I73" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03393-5?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/22/e0217252025</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Identifying novel metabolites in children with attention-deficit hyperactivity disorder through metabolome profiling</t>
+          <t>Dorsal–Caudal and Ventral Hippocampi Target Different Cell Populations in the Medial Frontal Cortex in Rodents</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03393-5</t>
+          <t>10.1523/JNEUROSCI.0217-25.2025</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Chi-Yung Shang</t>
+          <t>Shinya Ohara</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>cyshang@ntu.edu.tw</t>
+          <t>shinya.ohara.d3@tohoku.ac.jp</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I74" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -3577,6 +3801,9 @@
           <t>pattern</t>
         </is>
       </c>
+      <c r="I75" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3619,6 +3846,9 @@
           <t>pattern</t>
         </is>
       </c>
+      <c r="I76" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3661,73 +3891,79 @@
           <t>pattern</t>
         </is>
       </c>
+      <c r="I77" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00298-3?dgcid=raven_jbs_etoc_email</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Neuron</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Activity-dependent development of the body’s touch receptors</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>10.1016/j.neuron.2025.04.015</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>David D. Ginty</t>
+          <t>Adam Steel</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>['last_author']</t>
+          <t>['first_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>david_ginty@hms.harvard.edu</t>
+          <t>adamdanielsteel@gmail.com</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I78" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41398-025-03272-z?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
+          <t>https://www.jneurosci.org/content/45/23/e0028252025</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Translational Psychiatry</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Psychiatric and cognitive function in patients with serotonin producing neuroendocrine tumors</t>
+          <t>Relating Scene Memory and Perception Activity to Functional Properties, Networks, and Landmarks of Posterior Cerebral Cortex—A Probabilistic Atlas</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>10.1038/s41398-025-03272-z</t>
+          <t>10.1523/JNEUROSCI.0028-25.2025</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Froukje E. de Vries</t>
+          <t>Caroline E. Robertson</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3737,81 +3973,87 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>f.d.vries@nki.nl</t>
+          <t>cerw@dartmouth.edu</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I79" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.nature.com/articles/s41398-025-03390-8?utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41398_AWA1_GL_DTEC_054CI_TOC-250531&amp;utm_content=20250531</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Translational Psychiatry</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Computational mechanisms underlying multi-step planning deficits in methamphetamine use disorder</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1038/s41398-025-03390-8</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Marie-Lucie Read</t>
+          <t>Ryan Smith</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>readms2@cardiff.ac.uk</t>
+          <t>rsmith@laureateinstitute.org</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I80" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1700242025</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Multimodal MEG and Microstructure–MRI Investigations of the Human Hippocampal Scene Network</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1700-24.2025</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Andrew D. Lawrence</t>
+          <t>Stuart Berg</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3821,81 +4063,87 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Andrew.D.Lawrence@ed.ac.uk</t>
+          <t>bergs@janelia.hhmi.org</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I81" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Yan Chen</t>
+          <t>Gerald M. Rubin</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>['first_author', 'corresponding_author']</t>
+          <t>['corresponding_author']</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>chen_yan@hznu.edu.cn</t>
+          <t>rubing@janelia.hhmi.org</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I82" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://www.jneurosci.org/content/45/22/e1684242025</t>
+          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>The Journal of Neuroscience</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Clinical Diagnostic and Prognostic Value of Residual Language Learning Ability in Patients with Disorders of Consciousness</t>
+          <t>Connectome-driven neural inventory of a complete visual system</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>10.1523/JNEUROSCI.1684-24.2025</t>
+          <t>10.1038/s41586-025-08746-0</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Haibo Di</t>
+          <t>Michael B. Reiser</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3905,139 +4153,286 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>haibodi@hznu.edu.cn</t>
+          <t>reiserm@janelia.hhmi.org</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I83" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.jneurosci.org/content/45/23/e1920232025</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>The Journal of Neuroscience</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>Uncertainty, Not Mental Content, Drives Dorsomedial Prefrontal Engagement during Inferences about Others</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1523/JNEUROSCI.1920-23.2025</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Stuart Berg</t>
+          <t>Adrianna C. Jenkins</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author', 'corresponding_author']</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>bergs@janelia.hhmi.org</t>
+          <t>acjenk@upenn.edu</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I84" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.pnas.org/doi/10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Proceedings of the National Academy of Sciences</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>High-affinity detection of biotinylated endogenous neuroligin-1 at excitatory and inhibitory synapses using a tagged knock-in mouse</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1073/pnas.2411669122</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Gerald M. Rubin</t>
+          <t>Olivier Thoumine</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>['corresponding_author']</t>
+          <t>['last_author']</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>rubing@janelia.hhmi.org</t>
+          <t>olivier.thoumine@u-bordeaux.fr</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I85" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://www.nature.com/articles/s41586-025-08746-0?WT.ec_id=NATURE-20250529&amp;utm_source=nature_etoc&amp;utm_medium=email&amp;utm_campaign=CONR_41586_AWA1_GL_DTEC_054CI_TOC-250529</t>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Neuron</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Connectome-driven neural inventory of a complete visual system</t>
+          <t>A pontine center in descending pain control</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>10.1038/s41586-025-08746-0</t>
+          <t>10.1016/j.neuron.2025.02.028</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Michael B. Reiser</t>
+          <t>Wenjie Zhou</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>['last_author', 'corresponding_author']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>reiserm@janelia.hhmi.org</t>
+          <t>zhouwj2022@shsmu.edu.cn</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
           <t>pattern</t>
         </is>
+      </c>
+      <c r="I86" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Neuron</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>A pontine center in descending pain control</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>10.1016/j.neuron.2025.02.028</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Wenxi Huang</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>tw.huang@siat.ac.cn</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="I87" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Neuron</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>A pontine center in descending pain control</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>10.1016/j.neuron.2025.02.028</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Tianwen Huang</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>tw.huang@siat.ac.cn</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="I88" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>https://www.cell.com/neuron/fulltext/S0896-6273(25)00171-0?dgcid=raven_jbs_etoc_email</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Neuron</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>A pontine center in descending pain control</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>10.1016/j.neuron.2025.02.028</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Yuanyuan Liu</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>['last_author']</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>yuanyuan.liu@nih.gov</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>pattern</t>
+        </is>
+      </c>
+      <c r="I89" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>